<commit_message>
docs(asvs): update ASVS tracker statuses for file and authorization controls
</commit_message>
<xml_diff>
--- a/Deliverables/Phase1/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/Phase1/ASVS_5.0_Tracker.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabio\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ambiente de Trabalho\2º semestre\DESOFT\desofs2026-wed_nap_5\Deliverables\Phase1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66409195-AD97-4147-8138-5D92BEAE5132}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FFD66DE-621F-4BDB-864C-9D42EBD2FA94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="16" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" firstSheet="8" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2071" uniqueCount="906">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2103" uniqueCount="936">
   <si>
     <t>OWASP ASVS 5.0 – Compliance Tracker</t>
   </si>
@@ -2758,18 +2758,9 @@
     <t xml:space="preserve">SR11 </t>
   </si>
   <si>
-    <t>FR2</t>
-  </si>
-  <si>
     <t>Está previsto o sistema ter as roles Admin, professor e student</t>
   </si>
   <si>
-    <t>Está documentado em vários requisitos funcionais</t>
-  </si>
-  <si>
-    <t>FR8-18</t>
-  </si>
-  <si>
     <t xml:space="preserve">Chapter 13: Mitigations </t>
   </si>
   <si>
@@ -2783,6 +2774,105 @@
   </si>
   <si>
     <t>SR15</t>
+  </si>
+  <si>
+    <t>File validation requirements are defined, including allowed types, extensions, and size limits (SR11).</t>
+  </si>
+  <si>
+    <t>Maximum file size limits are enforced to prevent performance degradation and denial of service (SR11).</t>
+  </si>
+  <si>
+    <t>File extensions are validated on upload, including files contained within archives (SR11).</t>
+  </si>
+  <si>
+    <t>Compressed files are validated against maximum allowed uncompressed size to prevent resource exhaustion.</t>
+  </si>
+  <si>
+    <t>File size limits are enforced; upload quotas are considered as mitigation for storage abuse.</t>
+  </si>
+  <si>
+    <t>Compressed files containing unsafe elements such as symlinks are restricted or validated.</t>
+  </si>
+  <si>
+    <t>Uploaded files are validated to prevent oversized or malicious content causing resource exhaustion.</t>
+  </si>
+  <si>
+    <t>Files are stored outside public directories and are not executed as server-side code (SR8).</t>
+  </si>
+  <si>
+    <t>File paths are generated server-side, preventing usage of user-controlled filenames (SR12).</t>
+  </si>
+  <si>
+    <t>Server-side file processing ignores user-provided paths to prevent path traversal vulnerabilities (SR12).</t>
+  </si>
+  <si>
+    <t>User-submitted filenames are validated or ignored to prevent path traversal and injection attacks (SR12).</t>
+  </si>
+  <si>
+    <t>File names are sanitized and encoded before being returned in responses (SR10).</t>
+  </si>
+  <si>
+    <t>Files from untrusted sources are validated and may be scanned to prevent malicious content delivery.</t>
+  </si>
+  <si>
+    <t>Compliant</t>
+  </si>
+  <si>
+    <t>SR11</t>
+  </si>
+  <si>
+    <t>SR10</t>
+  </si>
+  <si>
+    <t>SR10, SR12</t>
+  </si>
+  <si>
+    <t>SR12</t>
+  </si>
+  <si>
+    <t>SR11, NFR13</t>
+  </si>
+  <si>
+    <t>NFR6</t>
+  </si>
+  <si>
+    <t>Authorization and authentication mechanisms are defined through RBAC and secure session/token handling.</t>
+  </si>
+  <si>
+    <t>FR2, SR4, SR5</t>
+  </si>
+  <si>
+    <t>FR8-18, SR4, SR5</t>
+  </si>
+  <si>
+    <t>Field-level and data access restrictions are partially defined through functional requirements and RBAC logic.</t>
+  </si>
+  <si>
+    <t>Access to data is restricted based on user role and course enrollment validation.</t>
+  </si>
+  <si>
+    <t>Function-level access is enforced through role-based access control (Admin, Professor, Student).</t>
+  </si>
+  <si>
+    <t>FR2, SR4</t>
+  </si>
+  <si>
+    <t>SR5, SR6</t>
+  </si>
+  <si>
+    <t>Authorization is enforced at the server-side API layer and does not rely on client-side controls.</t>
+  </si>
+  <si>
+    <t>SR4, SR5</t>
+  </si>
+  <si>
+    <t>Access control decisions are based on the authenticated user and ownership or enrollment relationships.</t>
+  </si>
+  <si>
+    <t>Administrative access is protected through RBAC and authentication mechanisms, with additional logging controls.</t>
+  </si>
+  <si>
+    <t>SR2, SR4, SR16</t>
   </si>
 </sst>
 </file>
@@ -2940,7 +3030,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3012,6 +3102,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3100,7 +3193,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="pt-BR"/>
+  <c:lang val="pt-PT"/>
   <c:roundedCorners val="0"/>
   <c:style val="2"/>
   <c:chart>
@@ -3248,7 +3341,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -3432,7 +3525,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -3797,7 +3890,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>0.23076923076923078</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -4346,13 +4439,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P23"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
     <col min="2" max="13" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
@@ -4372,7 +4465,7 @@
       <c r="O1" s="24"/>
       <c r="P1" s="24"/>
     </row>
-    <row r="2" spans="1:16" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="25"/>
       <c r="B2" s="25"/>
       <c r="C2" s="25"/>
@@ -4390,7 +4483,7 @@
       <c r="O2" s="25"/>
       <c r="P2" s="25"/>
     </row>
-    <row r="3" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="26"/>
       <c r="B3" s="26"/>
       <c r="C3" s="1"/>
@@ -4401,7 +4494,7 @@
       <c r="M3" s="1"/>
       <c r="O3" s="1"/>
     </row>
-    <row r="5" spans="1:16" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
@@ -4442,7 +4535,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
@@ -4491,7 +4584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
         <v>15</v>
       </c>
@@ -4540,7 +4633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>16</v>
       </c>
@@ -4589,7 +4682,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
         <v>17</v>
       </c>
@@ -4638,7 +4731,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>18</v>
       </c>
@@ -4650,22 +4743,22 @@
       </c>
       <c r="D10" s="4">
         <f>COUNTIFS('V5 - File Handling'!$F$2:$F$18,"Compliant",'V5 - File Handling'!$E$2:$E$18,1)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E10" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F10" s="4">
         <v>5</v>
       </c>
       <c r="G10" s="4">
         <f>COUNTIFS('V5 - File Handling'!$F$2:$F$18,"Compliant",'V5 - File Handling'!$E$2:$E$18,2)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="I10" s="4">
         <v>4</v>
@@ -4680,14 +4773,14 @@
       </c>
       <c r="L10" s="4">
         <f>COUNTIF('V5 - File Handling'!$F$2:$F$18,"Compliant")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M10" s="5">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+        <v>0.23076923076923078</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
         <v>19</v>
       </c>
@@ -4736,7 +4829,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
@@ -4785,7 +4878,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
         <v>21</v>
       </c>
@@ -4834,7 +4927,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>22</v>
       </c>
@@ -4881,7 +4974,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
         <v>24</v>
       </c>
@@ -4930,7 +5023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>25</v>
       </c>
@@ -4979,7 +5072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="6" t="s">
         <v>26</v>
       </c>
@@ -5028,7 +5121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>27</v>
       </c>
@@ -5077,7 +5170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="6" t="s">
         <v>28</v>
       </c>
@@ -5126,7 +5219,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
         <v>29</v>
       </c>
@@ -5175,7 +5268,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="6" t="s">
         <v>30</v>
       </c>
@@ -5222,7 +5315,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>31</v>
       </c>
@@ -5269,7 +5362,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="9" t="s">
         <v>32</v>
       </c>
@@ -5283,11 +5376,11 @@
       </c>
       <c r="D23" s="10">
         <f>SUM(D6:D22)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E23" s="11">
         <f>IFERROR(AVERAGE(E6:E22),"")</f>
-        <v>0</v>
+        <v>3.3333333333333333E-2</v>
       </c>
       <c r="F23" s="10">
         <f>SUM(F6:F22)</f>
@@ -5295,11 +5388,11 @@
       </c>
       <c r="G23" s="10">
         <f>SUM(G6:G22)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H23" s="11">
         <f>IFERROR(AVERAGE(H6:H22),"")</f>
-        <v>0</v>
+        <v>1.1764705882352941E-2</v>
       </c>
       <c r="I23" s="10">
         <f>SUM(I6:I22)</f>
@@ -5315,11 +5408,11 @@
       </c>
       <c r="L23" s="10">
         <f>SUM(L6:L22)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M23" s="11">
         <f>IFERROR(AVERAGE(M6:M22),"")</f>
-        <v>0</v>
+        <v>1.3574660633484163E-2</v>
       </c>
     </row>
   </sheetData>
@@ -5385,7 +5478,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:H10"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -5397,7 +5490,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -5423,7 +5516,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>490</v>
       </c>
@@ -5437,7 +5530,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>490</v>
       </c>
@@ -5459,7 +5552,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>490</v>
       </c>
@@ -5481,7 +5574,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>490</v>
       </c>
@@ -5503,7 +5596,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="13" t="s">
         <v>498</v>
       </c>
@@ -5517,7 +5610,7 @@
       <c r="G6" s="13"/>
       <c r="H6" s="13"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
         <v>498</v>
       </c>
@@ -5539,7 +5632,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="19" t="s">
         <v>498</v>
       </c>
@@ -5561,7 +5654,7 @@
       <c r="G8" s="21"/>
       <c r="H8" s="21"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
         <v>498</v>
       </c>
@@ -5583,7 +5676,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="19" t="s">
         <v>498</v>
       </c>
@@ -5631,7 +5724,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:H44"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -5643,7 +5736,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -5669,7 +5762,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>508</v>
       </c>
@@ -5683,7 +5776,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>508</v>
       </c>
@@ -5705,7 +5798,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>508</v>
       </c>
@@ -5727,7 +5820,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="13" t="s">
         <v>514</v>
       </c>
@@ -5741,7 +5834,7 @@
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="14" t="s">
         <v>514</v>
       </c>
@@ -5763,7 +5856,7 @@
       <c r="G6" s="16"/>
       <c r="H6" s="16"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="19" t="s">
         <v>514</v>
       </c>
@@ -5785,7 +5878,7 @@
       <c r="G7" s="21"/>
       <c r="H7" s="21"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="14" t="s">
         <v>514</v>
       </c>
@@ -5807,7 +5900,7 @@
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
     </row>
-    <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="13" t="s">
         <v>522</v>
       </c>
@@ -5821,7 +5914,7 @@
       <c r="G9" s="13"/>
       <c r="H9" s="13"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="14" t="s">
         <v>522</v>
       </c>
@@ -5843,7 +5936,7 @@
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="19" t="s">
         <v>522</v>
       </c>
@@ -5865,7 +5958,7 @@
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>522</v>
       </c>
@@ -5887,7 +5980,7 @@
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="19" t="s">
         <v>522</v>
       </c>
@@ -5909,7 +6002,7 @@
       <c r="G13" s="21"/>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="14" t="s">
         <v>522</v>
       </c>
@@ -5931,7 +6024,7 @@
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
     </row>
-    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="13" t="s">
         <v>534</v>
       </c>
@@ -5945,7 +6038,7 @@
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="14" t="s">
         <v>534</v>
       </c>
@@ -5967,7 +6060,7 @@
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="19" t="s">
         <v>534</v>
       </c>
@@ -5989,7 +6082,7 @@
       <c r="G17" s="21"/>
       <c r="H17" s="21"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="14" t="s">
         <v>534</v>
       </c>
@@ -6011,7 +6104,7 @@
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="19" t="s">
         <v>534</v>
       </c>
@@ -6033,7 +6126,7 @@
       <c r="G19" s="21"/>
       <c r="H19" s="21"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="14" t="s">
         <v>534</v>
       </c>
@@ -6055,7 +6148,7 @@
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="19" t="s">
         <v>534</v>
       </c>
@@ -6077,7 +6170,7 @@
       <c r="G21" s="21"/>
       <c r="H21" s="21"/>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="14" t="s">
         <v>534</v>
       </c>
@@ -6099,7 +6192,7 @@
       <c r="G22" s="16"/>
       <c r="H22" s="16"/>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="19" t="s">
         <v>534</v>
       </c>
@@ -6121,7 +6214,7 @@
       <c r="G23" s="21"/>
       <c r="H23" s="21"/>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="14" t="s">
         <v>534</v>
       </c>
@@ -6143,7 +6236,7 @@
       <c r="G24" s="16"/>
       <c r="H24" s="16"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="19" t="s">
         <v>534</v>
       </c>
@@ -6165,7 +6258,7 @@
       <c r="G25" s="21"/>
       <c r="H25" s="21"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="14" t="s">
         <v>534</v>
       </c>
@@ -6187,7 +6280,7 @@
       <c r="G26" s="16"/>
       <c r="H26" s="16"/>
     </row>
-    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="19" t="s">
         <v>534</v>
       </c>
@@ -6209,7 +6302,7 @@
       <c r="G27" s="21"/>
       <c r="H27" s="21"/>
     </row>
-    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="14" t="s">
         <v>534</v>
       </c>
@@ -6231,7 +6324,7 @@
       <c r="G28" s="16"/>
       <c r="H28" s="16"/>
     </row>
-    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="19" t="s">
         <v>534</v>
       </c>
@@ -6253,7 +6346,7 @@
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
     </row>
-    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="14" t="s">
         <v>534</v>
       </c>
@@ -6275,7 +6368,7 @@
       <c r="G30" s="16"/>
       <c r="H30" s="16"/>
     </row>
-    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="19" t="s">
         <v>534</v>
       </c>
@@ -6297,7 +6390,7 @@
       <c r="G31" s="21"/>
       <c r="H31" s="21"/>
     </row>
-    <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="13" t="s">
         <v>568</v>
       </c>
@@ -6311,7 +6404,7 @@
       <c r="G32" s="13"/>
       <c r="H32" s="13"/>
     </row>
-    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="14" t="s">
         <v>568</v>
       </c>
@@ -6333,7 +6426,7 @@
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
     </row>
-    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="19" t="s">
         <v>568</v>
       </c>
@@ -6355,7 +6448,7 @@
       <c r="G34" s="21"/>
       <c r="H34" s="21"/>
     </row>
-    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="14" t="s">
         <v>568</v>
       </c>
@@ -6377,7 +6470,7 @@
       <c r="G35" s="16"/>
       <c r="H35" s="16"/>
     </row>
-    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="19" t="s">
         <v>568</v>
       </c>
@@ -6399,7 +6492,7 @@
       <c r="G36" s="21"/>
       <c r="H36" s="21"/>
     </row>
-    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="14" t="s">
         <v>568</v>
       </c>
@@ -6421,7 +6514,7 @@
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
     </row>
-    <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="13" t="s">
         <v>580</v>
       </c>
@@ -6435,7 +6528,7 @@
       <c r="G38" s="13"/>
       <c r="H38" s="13"/>
     </row>
-    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="14" t="s">
         <v>580</v>
       </c>
@@ -6457,7 +6550,7 @@
       <c r="G39" s="16"/>
       <c r="H39" s="16"/>
     </row>
-    <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="19" t="s">
         <v>580</v>
       </c>
@@ -6479,7 +6572,7 @@
       <c r="G40" s="21"/>
       <c r="H40" s="21"/>
     </row>
-    <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="13" t="s">
         <v>586</v>
       </c>
@@ -6493,7 +6586,7 @@
       <c r="G41" s="13"/>
       <c r="H41" s="13"/>
     </row>
-    <row r="42" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="14" t="s">
         <v>586</v>
       </c>
@@ -6515,7 +6608,7 @@
       <c r="G42" s="16"/>
       <c r="H42" s="16"/>
     </row>
-    <row r="43" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="19" t="s">
         <v>586</v>
       </c>
@@ -6537,7 +6630,7 @@
       <c r="G43" s="21"/>
       <c r="H43" s="21"/>
     </row>
-    <row r="44" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="14" t="s">
         <v>586</v>
       </c>
@@ -6585,7 +6678,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:H32"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -6597,7 +6690,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -6623,7 +6716,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>594</v>
       </c>
@@ -6637,7 +6730,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>594</v>
       </c>
@@ -6659,7 +6752,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>594</v>
       </c>
@@ -6681,7 +6774,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>594</v>
       </c>
@@ -6703,7 +6796,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>594</v>
       </c>
@@ -6725,7 +6818,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="13" t="s">
         <v>604</v>
       </c>
@@ -6739,7 +6832,7 @@
       <c r="G7" s="13"/>
       <c r="H7" s="13"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="14" t="s">
         <v>604</v>
       </c>
@@ -6761,7 +6854,7 @@
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="19" t="s">
         <v>604</v>
       </c>
@@ -6783,7 +6876,7 @@
       <c r="G9" s="21"/>
       <c r="H9" s="21"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="14" t="s">
         <v>604</v>
       </c>
@@ -6805,7 +6898,7 @@
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="19" t="s">
         <v>604</v>
       </c>
@@ -6827,7 +6920,7 @@
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>604</v>
       </c>
@@ -6849,7 +6942,7 @@
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="13" t="s">
         <v>616</v>
       </c>
@@ -6863,7 +6956,7 @@
       <c r="G13" s="13"/>
       <c r="H13" s="13"/>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="14" t="s">
         <v>616</v>
       </c>
@@ -6885,7 +6978,7 @@
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="19" t="s">
         <v>616</v>
       </c>
@@ -6907,7 +7000,7 @@
       <c r="G15" s="21"/>
       <c r="H15" s="21"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="14" t="s">
         <v>616</v>
       </c>
@@ -6929,7 +7022,7 @@
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="19" t="s">
         <v>616</v>
       </c>
@@ -6951,7 +7044,7 @@
       <c r="G17" s="21"/>
       <c r="H17" s="21"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="14" t="s">
         <v>616</v>
       </c>
@@ -6973,7 +7066,7 @@
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
     </row>
-    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="13" t="s">
         <v>628</v>
       </c>
@@ -6987,7 +7080,7 @@
       <c r="G19" s="13"/>
       <c r="H19" s="13"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="14" t="s">
         <v>628</v>
       </c>
@@ -7009,7 +7102,7 @@
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="19" t="s">
         <v>628</v>
       </c>
@@ -7031,7 +7124,7 @@
       <c r="G21" s="21"/>
       <c r="H21" s="21"/>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="14" t="s">
         <v>628</v>
       </c>
@@ -7053,7 +7146,7 @@
       <c r="G22" s="16"/>
       <c r="H22" s="16"/>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="19" t="s">
         <v>628</v>
       </c>
@@ -7075,7 +7168,7 @@
       <c r="G23" s="21"/>
       <c r="H23" s="21"/>
     </row>
-    <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="13" t="s">
         <v>638</v>
       </c>
@@ -7089,7 +7182,7 @@
       <c r="G24" s="13"/>
       <c r="H24" s="13"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="14" t="s">
         <v>638</v>
       </c>
@@ -7111,7 +7204,7 @@
       <c r="G25" s="16"/>
       <c r="H25" s="16"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="19" t="s">
         <v>638</v>
       </c>
@@ -7133,7 +7226,7 @@
       <c r="G26" s="21"/>
       <c r="H26" s="21"/>
     </row>
-    <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="13" t="s">
         <v>644</v>
       </c>
@@ -7147,7 +7240,7 @@
       <c r="G27" s="13"/>
       <c r="H27" s="13"/>
     </row>
-    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="14" t="s">
         <v>644</v>
       </c>
@@ -7169,7 +7262,7 @@
       <c r="G28" s="16"/>
       <c r="H28" s="16"/>
     </row>
-    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="19" t="s">
         <v>644</v>
       </c>
@@ -7191,7 +7284,7 @@
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
     </row>
-    <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="13" t="s">
         <v>650</v>
       </c>
@@ -7205,7 +7298,7 @@
       <c r="G30" s="13"/>
       <c r="H30" s="13"/>
     </row>
-    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="14" t="s">
         <v>650</v>
       </c>
@@ -7227,7 +7320,7 @@
       <c r="G31" s="16"/>
       <c r="H31" s="16"/>
     </row>
-    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="19" t="s">
         <v>650</v>
       </c>
@@ -7275,7 +7368,7 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -7287,7 +7380,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -7313,7 +7406,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>656</v>
       </c>
@@ -7327,7 +7420,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>656</v>
       </c>
@@ -7349,7 +7442,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>656</v>
       </c>
@@ -7371,7 +7464,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>656</v>
       </c>
@@ -7393,7 +7486,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>656</v>
       </c>
@@ -7415,7 +7508,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
         <v>656</v>
       </c>
@@ -7437,7 +7530,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="13" t="s">
         <v>668</v>
       </c>
@@ -7451,7 +7544,7 @@
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
         <v>668</v>
       </c>
@@ -7473,7 +7566,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="19" t="s">
         <v>668</v>
       </c>
@@ -7495,7 +7588,7 @@
       <c r="G10" s="21"/>
       <c r="H10" s="21"/>
     </row>
-    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
         <v>674</v>
       </c>
@@ -7509,7 +7602,7 @@
       <c r="G11" s="13"/>
       <c r="H11" s="13"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>674</v>
       </c>
@@ -7531,7 +7624,7 @@
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="19" t="s">
         <v>674</v>
       </c>
@@ -7553,7 +7646,7 @@
       <c r="G13" s="21"/>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="14" t="s">
         <v>674</v>
       </c>
@@ -7575,7 +7668,7 @@
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="19" t="s">
         <v>674</v>
       </c>
@@ -7597,7 +7690,7 @@
       <c r="G15" s="21"/>
       <c r="H15" s="21"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="14" t="s">
         <v>674</v>
       </c>
@@ -7645,7 +7738,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:H26"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -7657,7 +7750,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -7683,7 +7776,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>686</v>
       </c>
@@ -7697,7 +7790,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>686</v>
       </c>
@@ -7719,7 +7812,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>686</v>
       </c>
@@ -7741,7 +7834,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>686</v>
       </c>
@@ -7763,7 +7856,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>686</v>
       </c>
@@ -7785,7 +7878,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="13" t="s">
         <v>696</v>
       </c>
@@ -7799,7 +7892,7 @@
       <c r="G7" s="13"/>
       <c r="H7" s="13"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="14" t="s">
         <v>696</v>
       </c>
@@ -7821,7 +7914,7 @@
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="19" t="s">
         <v>696</v>
       </c>
@@ -7843,7 +7936,7 @@
       <c r="G9" s="21"/>
       <c r="H9" s="21"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="14" t="s">
         <v>696</v>
       </c>
@@ -7865,7 +7958,7 @@
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="19" t="s">
         <v>696</v>
       </c>
@@ -7887,7 +7980,7 @@
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>696</v>
       </c>
@@ -7909,7 +8002,7 @@
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="19" t="s">
         <v>696</v>
       </c>
@@ -7931,7 +8024,7 @@
       <c r="G13" s="21"/>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="13" t="s">
         <v>710</v>
       </c>
@@ -7945,7 +8038,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
         <v>710</v>
       </c>
@@ -7967,7 +8060,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>710</v>
       </c>
@@ -7989,7 +8082,7 @@
       <c r="G16" s="21"/>
       <c r="H16" s="21"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="14" t="s">
         <v>710</v>
       </c>
@@ -8011,7 +8104,7 @@
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="19" t="s">
         <v>710</v>
       </c>
@@ -8033,7 +8126,7 @@
       <c r="G18" s="21"/>
       <c r="H18" s="21"/>
     </row>
-    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="13" t="s">
         <v>720</v>
       </c>
@@ -8047,7 +8140,7 @@
       <c r="G19" s="13"/>
       <c r="H19" s="13"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="14" t="s">
         <v>720</v>
       </c>
@@ -8069,7 +8162,7 @@
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="19" t="s">
         <v>720</v>
       </c>
@@ -8091,7 +8184,7 @@
       <c r="G21" s="21"/>
       <c r="H21" s="21"/>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="14" t="s">
         <v>720</v>
       </c>
@@ -8113,7 +8206,7 @@
       <c r="G22" s="16"/>
       <c r="H22" s="16"/>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="19" t="s">
         <v>720</v>
       </c>
@@ -8135,7 +8228,7 @@
       <c r="G23" s="21"/>
       <c r="H23" s="21"/>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="14" t="s">
         <v>720</v>
       </c>
@@ -8157,7 +8250,7 @@
       <c r="G24" s="16"/>
       <c r="H24" s="16"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="19" t="s">
         <v>720</v>
       </c>
@@ -8179,7 +8272,7 @@
       <c r="G25" s="21"/>
       <c r="H25" s="21"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="14" t="s">
         <v>720</v>
       </c>
@@ -8227,7 +8320,7 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:H17"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -8239,7 +8332,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -8265,7 +8358,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>736</v>
       </c>
@@ -8279,7 +8372,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>736</v>
       </c>
@@ -8300,10 +8393,10 @@
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16" t="s">
-        <v>904</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>901</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>736</v>
       </c>
@@ -8324,10 +8417,10 @@
       </c>
       <c r="G4" s="21"/>
       <c r="H4" s="21" t="s">
-        <v>901</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="13" t="s">
         <v>742</v>
       </c>
@@ -8341,7 +8434,7 @@
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="14" t="s">
         <v>742</v>
       </c>
@@ -8363,7 +8456,7 @@
       <c r="G6" s="16"/>
       <c r="H6" s="16"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="19" t="s">
         <v>742</v>
       </c>
@@ -8385,7 +8478,7 @@
       <c r="G7" s="21"/>
       <c r="H7" s="21"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="14" t="s">
         <v>742</v>
       </c>
@@ -8407,7 +8500,7 @@
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="19" t="s">
         <v>742</v>
       </c>
@@ -8429,7 +8522,7 @@
       <c r="G9" s="21"/>
       <c r="H9" s="21"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="14" t="s">
         <v>742</v>
       </c>
@@ -8451,7 +8544,7 @@
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="19" t="s">
         <v>742</v>
       </c>
@@ -8473,7 +8566,7 @@
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>742</v>
       </c>
@@ -8495,7 +8588,7 @@
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="19" t="s">
         <v>742</v>
       </c>
@@ -8517,7 +8610,7 @@
       <c r="G13" s="21"/>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="13" t="s">
         <v>760</v>
       </c>
@@ -8531,7 +8624,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
         <v>760</v>
       </c>
@@ -8553,7 +8646,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>760</v>
       </c>
@@ -8575,7 +8668,7 @@
       <c r="G16" s="21"/>
       <c r="H16" s="21"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="14" t="s">
         <v>760</v>
       </c>
@@ -8623,7 +8716,7 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:H26"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -8635,7 +8728,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -8661,7 +8754,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>768</v>
       </c>
@@ -8675,7 +8768,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>768</v>
       </c>
@@ -8696,10 +8789,10 @@
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16" t="s">
-        <v>905</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>768</v>
       </c>
@@ -8721,7 +8814,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>768</v>
       </c>
@@ -8743,7 +8836,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>768</v>
       </c>
@@ -8765,7 +8858,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
         <v>768</v>
       </c>
@@ -8787,7 +8880,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="13" t="s">
         <v>780</v>
       </c>
@@ -8801,7 +8894,7 @@
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
         <v>780</v>
       </c>
@@ -8823,7 +8916,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="19" t="s">
         <v>780</v>
       </c>
@@ -8845,7 +8938,7 @@
       <c r="G10" s="21"/>
       <c r="H10" s="21"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="14" t="s">
         <v>780</v>
       </c>
@@ -8867,7 +8960,7 @@
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="19" t="s">
         <v>780</v>
       </c>
@@ -8889,7 +8982,7 @@
       <c r="G12" s="21"/>
       <c r="H12" s="21"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
         <v>780</v>
       </c>
@@ -8911,7 +9004,7 @@
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="13" t="s">
         <v>792</v>
       </c>
@@ -8925,7 +9018,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
         <v>792</v>
       </c>
@@ -8947,7 +9040,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>792</v>
       </c>
@@ -8969,7 +9062,7 @@
       <c r="G16" s="21"/>
       <c r="H16" s="21"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="14" t="s">
         <v>792</v>
       </c>
@@ -8991,7 +9084,7 @@
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="19" t="s">
         <v>792</v>
       </c>
@@ -9013,7 +9106,7 @@
       <c r="G18" s="21"/>
       <c r="H18" s="21"/>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="14" t="s">
         <v>792</v>
       </c>
@@ -9035,7 +9128,7 @@
       <c r="G19" s="16"/>
       <c r="H19" s="16"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="19" t="s">
         <v>792</v>
       </c>
@@ -9057,7 +9150,7 @@
       <c r="G20" s="21"/>
       <c r="H20" s="21"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="14" t="s">
         <v>792</v>
       </c>
@@ -9079,7 +9172,7 @@
       <c r="G21" s="16"/>
       <c r="H21" s="16"/>
     </row>
-    <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="13" t="s">
         <v>808</v>
       </c>
@@ -9093,7 +9186,7 @@
       <c r="G22" s="13"/>
       <c r="H22" s="13"/>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="14" t="s">
         <v>808</v>
       </c>
@@ -9115,7 +9208,7 @@
       <c r="G23" s="16"/>
       <c r="H23" s="16"/>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="19" t="s">
         <v>808</v>
       </c>
@@ -9137,7 +9230,7 @@
       <c r="G24" s="21"/>
       <c r="H24" s="21"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="14" t="s">
         <v>808</v>
       </c>
@@ -9159,7 +9252,7 @@
       <c r="G25" s="16"/>
       <c r="H25" s="16"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="19" t="s">
         <v>808</v>
       </c>
@@ -9207,7 +9300,7 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="A1:H23"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -9219,7 +9312,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -9245,7 +9338,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>818</v>
       </c>
@@ -9259,7 +9352,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>818</v>
       </c>
@@ -9281,7 +9374,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="13" t="s">
         <v>822</v>
       </c>
@@ -9295,7 +9388,7 @@
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>822</v>
       </c>
@@ -9317,7 +9410,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>822</v>
       </c>
@@ -9339,7 +9432,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
         <v>822</v>
       </c>
@@ -9361,7 +9454,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="19" t="s">
         <v>822</v>
       </c>
@@ -9383,7 +9476,7 @@
       <c r="G8" s="21"/>
       <c r="H8" s="21"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
         <v>822</v>
       </c>
@@ -9405,7 +9498,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="13" t="s">
         <v>834</v>
       </c>
@@ -9419,7 +9512,7 @@
       <c r="G10" s="13"/>
       <c r="H10" s="13"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="14" t="s">
         <v>834</v>
       </c>
@@ -9441,7 +9534,7 @@
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="19" t="s">
         <v>834</v>
       </c>
@@ -9463,7 +9556,7 @@
       <c r="G12" s="21"/>
       <c r="H12" s="21"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
         <v>834</v>
       </c>
@@ -9485,7 +9578,7 @@
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="19" t="s">
         <v>834</v>
       </c>
@@ -9507,7 +9600,7 @@
       <c r="G14" s="21"/>
       <c r="H14" s="21"/>
     </row>
-    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="13" t="s">
         <v>844</v>
       </c>
@@ -9521,7 +9614,7 @@
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="14" t="s">
         <v>844</v>
       </c>
@@ -9543,7 +9636,7 @@
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="19" t="s">
         <v>844</v>
       </c>
@@ -9565,7 +9658,7 @@
       <c r="G17" s="21"/>
       <c r="H17" s="21"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="14" t="s">
         <v>844</v>
       </c>
@@ -9587,7 +9680,7 @@
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
     </row>
-    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="13" t="s">
         <v>852</v>
       </c>
@@ -9601,7 +9694,7 @@
       <c r="G19" s="13"/>
       <c r="H19" s="13"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="14" t="s">
         <v>852</v>
       </c>
@@ -9623,7 +9716,7 @@
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="19" t="s">
         <v>852</v>
       </c>
@@ -9645,7 +9738,7 @@
       <c r="G21" s="21"/>
       <c r="H21" s="21"/>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="14" t="s">
         <v>852</v>
       </c>
@@ -9667,7 +9760,7 @@
       <c r="G22" s="16"/>
       <c r="H22" s="16"/>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="19" t="s">
         <v>852</v>
       </c>
@@ -9715,7 +9808,7 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -9727,7 +9820,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -9753,7 +9846,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>862</v>
       </c>
@@ -9767,7 +9860,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>862</v>
       </c>
@@ -9789,7 +9882,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>862</v>
       </c>
@@ -9811,7 +9904,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="13" t="s">
         <v>868</v>
       </c>
@@ -9825,7 +9918,7 @@
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="14" t="s">
         <v>868</v>
       </c>
@@ -9847,7 +9940,7 @@
       <c r="G6" s="16"/>
       <c r="H6" s="16"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="19" t="s">
         <v>868</v>
       </c>
@@ -9869,7 +9962,7 @@
       <c r="G7" s="21"/>
       <c r="H7" s="21"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="14" t="s">
         <v>868</v>
       </c>
@@ -9891,7 +9984,7 @@
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="19" t="s">
         <v>868</v>
       </c>
@@ -9913,7 +10006,7 @@
       <c r="G9" s="21"/>
       <c r="H9" s="21"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="14" t="s">
         <v>868</v>
       </c>
@@ -9935,7 +10028,7 @@
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="19" t="s">
         <v>868</v>
       </c>
@@ -9957,7 +10050,7 @@
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>868</v>
       </c>
@@ -9979,7 +10072,7 @@
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="19" t="s">
         <v>868</v>
       </c>
@@ -10001,7 +10094,7 @@
       <c r="G13" s="21"/>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="13" t="s">
         <v>886</v>
       </c>
@@ -10015,7 +10108,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
         <v>886</v>
       </c>
@@ -10037,7 +10130,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>886</v>
       </c>
@@ -10085,7 +10178,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H36"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -10097,7 +10190,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -10123,7 +10216,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>41</v>
       </c>
@@ -10137,7 +10230,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>41</v>
       </c>
@@ -10159,7 +10252,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>41</v>
       </c>
@@ -10181,7 +10274,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="13" t="s">
         <v>48</v>
       </c>
@@ -10195,7 +10288,7 @@
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="14" t="s">
         <v>48</v>
       </c>
@@ -10217,7 +10310,7 @@
       <c r="G6" s="16"/>
       <c r="H6" s="16"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="19" t="s">
         <v>48</v>
       </c>
@@ -10239,7 +10332,7 @@
       <c r="G7" s="21"/>
       <c r="H7" s="21"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="14" t="s">
         <v>48</v>
       </c>
@@ -10261,7 +10354,7 @@
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="19" t="s">
         <v>48</v>
       </c>
@@ -10283,7 +10376,7 @@
       <c r="G9" s="21"/>
       <c r="H9" s="21"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="14" t="s">
         <v>48</v>
       </c>
@@ -10305,7 +10398,7 @@
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="19" t="s">
         <v>48</v>
       </c>
@@ -10327,7 +10420,7 @@
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>48</v>
       </c>
@@ -10349,7 +10442,7 @@
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="19" t="s">
         <v>48</v>
       </c>
@@ -10371,7 +10464,7 @@
       <c r="G13" s="21"/>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="14" t="s">
         <v>48</v>
       </c>
@@ -10393,7 +10486,7 @@
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="19" t="s">
         <v>48</v>
       </c>
@@ -10415,7 +10508,7 @@
       <c r="G15" s="21"/>
       <c r="H15" s="21"/>
     </row>
-    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="13" t="s">
         <v>70</v>
       </c>
@@ -10429,7 +10522,7 @@
       <c r="G16" s="13"/>
       <c r="H16" s="13"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="14" t="s">
         <v>70</v>
       </c>
@@ -10451,7 +10544,7 @@
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="19" t="s">
         <v>70</v>
       </c>
@@ -10473,7 +10566,7 @@
       <c r="G18" s="21"/>
       <c r="H18" s="21"/>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="14" t="s">
         <v>70</v>
       </c>
@@ -10495,7 +10588,7 @@
       <c r="G19" s="16"/>
       <c r="H19" s="16"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="19" t="s">
         <v>70</v>
       </c>
@@ -10517,7 +10610,7 @@
       <c r="G20" s="21"/>
       <c r="H20" s="21"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="14" t="s">
         <v>70</v>
       </c>
@@ -10539,7 +10632,7 @@
       <c r="G21" s="16"/>
       <c r="H21" s="16"/>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="19" t="s">
         <v>70</v>
       </c>
@@ -10561,7 +10654,7 @@
       <c r="G22" s="21"/>
       <c r="H22" s="21"/>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="14" t="s">
         <v>70</v>
       </c>
@@ -10583,7 +10676,7 @@
       <c r="G23" s="16"/>
       <c r="H23" s="16"/>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="19" t="s">
         <v>70</v>
       </c>
@@ -10605,7 +10698,7 @@
       <c r="G24" s="21"/>
       <c r="H24" s="21"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="14" t="s">
         <v>70</v>
       </c>
@@ -10627,7 +10720,7 @@
       <c r="G25" s="16"/>
       <c r="H25" s="16"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="19" t="s">
         <v>70</v>
       </c>
@@ -10649,7 +10742,7 @@
       <c r="G26" s="21"/>
       <c r="H26" s="21"/>
     </row>
-    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="14" t="s">
         <v>70</v>
       </c>
@@ -10671,7 +10764,7 @@
       <c r="G27" s="16"/>
       <c r="H27" s="16"/>
     </row>
-    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="19" t="s">
         <v>70</v>
       </c>
@@ -10693,7 +10786,7 @@
       <c r="G28" s="21"/>
       <c r="H28" s="21"/>
     </row>
-    <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="13" t="s">
         <v>96</v>
       </c>
@@ -10707,7 +10800,7 @@
       <c r="G29" s="13"/>
       <c r="H29" s="13"/>
     </row>
-    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="14" t="s">
         <v>96</v>
       </c>
@@ -10729,7 +10822,7 @@
       <c r="G30" s="16"/>
       <c r="H30" s="16"/>
     </row>
-    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="19" t="s">
         <v>96</v>
       </c>
@@ -10751,7 +10844,7 @@
       <c r="G31" s="21"/>
       <c r="H31" s="21"/>
     </row>
-    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="14" t="s">
         <v>96</v>
       </c>
@@ -10773,7 +10866,7 @@
       <c r="G32" s="16"/>
       <c r="H32" s="16"/>
     </row>
-    <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="13" t="s">
         <v>104</v>
       </c>
@@ -10787,7 +10880,7 @@
       <c r="G33" s="13"/>
       <c r="H33" s="13"/>
     </row>
-    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="14" t="s">
         <v>104</v>
       </c>
@@ -10809,7 +10902,7 @@
       <c r="G34" s="16"/>
       <c r="H34" s="16"/>
     </row>
-    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="19" t="s">
         <v>104</v>
       </c>
@@ -10831,7 +10924,7 @@
       <c r="G35" s="21"/>
       <c r="H35" s="21"/>
     </row>
-    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="14" t="s">
         <v>104</v>
       </c>
@@ -10879,7 +10972,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -10891,7 +10984,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -10917,7 +11010,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>112</v>
       </c>
@@ -10931,7 +11024,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>112</v>
       </c>
@@ -10955,7 +11048,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>112</v>
       </c>
@@ -10977,7 +11070,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>112</v>
       </c>
@@ -10999,7 +11092,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="13" t="s">
         <v>120</v>
       </c>
@@ -11013,7 +11106,7 @@
       <c r="G6" s="13"/>
       <c r="H6" s="13"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
         <v>120</v>
       </c>
@@ -11035,7 +11128,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="19" t="s">
         <v>120</v>
       </c>
@@ -11057,7 +11150,7 @@
       <c r="G8" s="21"/>
       <c r="H8" s="21"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
         <v>120</v>
       </c>
@@ -11079,7 +11172,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="13" t="s">
         <v>128</v>
       </c>
@@ -11093,7 +11186,7 @@
       <c r="G10" s="13"/>
       <c r="H10" s="13"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="14" t="s">
         <v>128</v>
       </c>
@@ -11115,7 +11208,7 @@
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="19" t="s">
         <v>128</v>
       </c>
@@ -11137,7 +11230,7 @@
       <c r="G12" s="21"/>
       <c r="H12" s="21"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
         <v>128</v>
       </c>
@@ -11159,7 +11252,7 @@
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="19" t="s">
         <v>128</v>
       </c>
@@ -11181,7 +11274,7 @@
       <c r="G14" s="21"/>
       <c r="H14" s="21"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
         <v>128</v>
       </c>
@@ -11203,7 +11296,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="13" t="s">
         <v>140</v>
       </c>
@@ -11217,7 +11310,7 @@
       <c r="G16" s="13"/>
       <c r="H16" s="13"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="14" t="s">
         <v>140</v>
       </c>
@@ -11239,7 +11332,7 @@
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="19" t="s">
         <v>140</v>
       </c>
@@ -11287,7 +11380,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H39"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -11299,7 +11392,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -11325,7 +11418,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>146</v>
       </c>
@@ -11339,7 +11432,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>146</v>
       </c>
@@ -11363,7 +11456,7 @@
       </c>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="13" t="s">
         <v>150</v>
       </c>
@@ -11377,7 +11470,7 @@
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>150</v>
       </c>
@@ -11399,7 +11492,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>150</v>
       </c>
@@ -11421,7 +11514,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
         <v>150</v>
       </c>
@@ -11443,7 +11536,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="13" t="s">
         <v>158</v>
       </c>
@@ -11457,7 +11550,7 @@
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
         <v>158</v>
       </c>
@@ -11479,7 +11572,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="19" t="s">
         <v>158</v>
       </c>
@@ -11501,7 +11594,7 @@
       <c r="G10" s="21"/>
       <c r="H10" s="21"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="14" t="s">
         <v>158</v>
       </c>
@@ -11523,7 +11616,7 @@
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="19" t="s">
         <v>158</v>
       </c>
@@ -11545,7 +11638,7 @@
       <c r="G12" s="21"/>
       <c r="H12" s="21"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
         <v>158</v>
       </c>
@@ -11567,7 +11660,7 @@
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="13" t="s">
         <v>170</v>
       </c>
@@ -11581,7 +11674,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
         <v>170</v>
       </c>
@@ -11603,7 +11696,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>170</v>
       </c>
@@ -11625,7 +11718,7 @@
       <c r="G16" s="21"/>
       <c r="H16" s="21"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="14" t="s">
         <v>170</v>
       </c>
@@ -11647,7 +11740,7 @@
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="19" t="s">
         <v>170</v>
       </c>
@@ -11669,7 +11762,7 @@
       <c r="G18" s="21"/>
       <c r="H18" s="21"/>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="14" t="s">
         <v>170</v>
       </c>
@@ -11691,7 +11784,7 @@
       <c r="G19" s="16"/>
       <c r="H19" s="16"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="19" t="s">
         <v>170</v>
       </c>
@@ -11713,7 +11806,7 @@
       <c r="G20" s="21"/>
       <c r="H20" s="21"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="14" t="s">
         <v>170</v>
       </c>
@@ -11735,7 +11828,7 @@
       <c r="G21" s="16"/>
       <c r="H21" s="16"/>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="19" t="s">
         <v>170</v>
       </c>
@@ -11757,7 +11850,7 @@
       <c r="G22" s="21"/>
       <c r="H22" s="21"/>
     </row>
-    <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="13" t="s">
         <v>188</v>
       </c>
@@ -11771,7 +11864,7 @@
       <c r="G23" s="13"/>
       <c r="H23" s="13"/>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="14" t="s">
         <v>188</v>
       </c>
@@ -11793,7 +11886,7 @@
       <c r="G24" s="16"/>
       <c r="H24" s="16"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="19" t="s">
         <v>188</v>
       </c>
@@ -11815,7 +11908,7 @@
       <c r="G25" s="21"/>
       <c r="H25" s="21"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="14" t="s">
         <v>188</v>
       </c>
@@ -11837,7 +11930,7 @@
       <c r="G26" s="16"/>
       <c r="H26" s="16"/>
     </row>
-    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="19" t="s">
         <v>188</v>
       </c>
@@ -11859,7 +11952,7 @@
       <c r="G27" s="21"/>
       <c r="H27" s="21"/>
     </row>
-    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="14" t="s">
         <v>188</v>
       </c>
@@ -11881,7 +11974,7 @@
       <c r="G28" s="16"/>
       <c r="H28" s="16"/>
     </row>
-    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="19" t="s">
         <v>188</v>
       </c>
@@ -11903,7 +11996,7 @@
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
     </row>
-    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="14" t="s">
         <v>188</v>
       </c>
@@ -11925,7 +12018,7 @@
       <c r="G30" s="16"/>
       <c r="H30" s="16"/>
     </row>
-    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="19" t="s">
         <v>188</v>
       </c>
@@ -11947,7 +12040,7 @@
       <c r="G31" s="21"/>
       <c r="H31" s="21"/>
     </row>
-    <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="13" t="s">
         <v>206</v>
       </c>
@@ -11961,7 +12054,7 @@
       <c r="G32" s="13"/>
       <c r="H32" s="13"/>
     </row>
-    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="14" t="s">
         <v>206</v>
       </c>
@@ -11983,7 +12076,7 @@
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
     </row>
-    <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="13" t="s">
         <v>210</v>
       </c>
@@ -11997,7 +12090,7 @@
       <c r="G34" s="13"/>
       <c r="H34" s="13"/>
     </row>
-    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="14" t="s">
         <v>210</v>
       </c>
@@ -12019,7 +12112,7 @@
       <c r="G35" s="16"/>
       <c r="H35" s="16"/>
     </row>
-    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="19" t="s">
         <v>210</v>
       </c>
@@ -12041,7 +12134,7 @@
       <c r="G36" s="21"/>
       <c r="H36" s="21"/>
     </row>
-    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="14" t="s">
         <v>210</v>
       </c>
@@ -12063,7 +12156,7 @@
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
     </row>
-    <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="19" t="s">
         <v>210</v>
       </c>
@@ -12085,7 +12178,7 @@
       <c r="G38" s="21"/>
       <c r="H38" s="21"/>
     </row>
-    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="14" t="s">
         <v>210</v>
       </c>
@@ -12133,7 +12226,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -12145,7 +12238,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -12171,7 +12264,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>222</v>
       </c>
@@ -12185,7 +12278,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>222</v>
       </c>
@@ -12207,7 +12300,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>222</v>
       </c>
@@ -12229,7 +12322,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>222</v>
       </c>
@@ -12251,7 +12344,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>222</v>
       </c>
@@ -12273,7 +12366,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
         <v>222</v>
       </c>
@@ -12295,7 +12388,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="13" t="s">
         <v>234</v>
       </c>
@@ -12309,7 +12402,7 @@
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
         <v>234</v>
       </c>
@@ -12331,7 +12424,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="19" t="s">
         <v>234</v>
       </c>
@@ -12353,7 +12446,7 @@
       <c r="G10" s="21"/>
       <c r="H10" s="21"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="14" t="s">
         <v>234</v>
       </c>
@@ -12375,7 +12468,7 @@
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="19" t="s">
         <v>234</v>
       </c>
@@ -12397,7 +12490,7 @@
       <c r="G12" s="21"/>
       <c r="H12" s="21"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
         <v>234</v>
       </c>
@@ -12419,7 +12512,7 @@
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="13" t="s">
         <v>246</v>
       </c>
@@ -12433,7 +12526,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
         <v>246</v>
       </c>
@@ -12455,7 +12548,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>246</v>
       </c>
@@ -12477,7 +12570,7 @@
       <c r="G16" s="21"/>
       <c r="H16" s="21"/>
     </row>
-    <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="13" t="s">
         <v>252</v>
       </c>
@@ -12491,7 +12584,7 @@
       <c r="G17" s="13"/>
       <c r="H17" s="13"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="14" t="s">
         <v>252</v>
       </c>
@@ -12513,7 +12606,7 @@
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="19" t="s">
         <v>252</v>
       </c>
@@ -12535,7 +12628,7 @@
       <c r="G19" s="21"/>
       <c r="H19" s="21"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="14" t="s">
         <v>252</v>
       </c>
@@ -12557,7 +12650,7 @@
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="19" t="s">
         <v>252</v>
       </c>
@@ -12605,7 +12698,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -12617,7 +12710,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -12643,7 +12736,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>262</v>
       </c>
@@ -12657,7 +12750,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>262</v>
       </c>
@@ -12674,14 +12767,16 @@
         <v>2</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>892</v>
-      </c>
-      <c r="G3" s="16"/>
+        <v>916</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>903</v>
+      </c>
       <c r="H3" s="16" t="s">
         <v>896</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="13" t="s">
         <v>266</v>
       </c>
@@ -12695,7 +12790,7 @@
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>266</v>
       </c>
@@ -12712,12 +12807,14 @@
         <v>1</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G5" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>904</v>
+      </c>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>266</v>
       </c>
@@ -12734,12 +12831,16 @@
         <v>1</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G6" s="21"/>
-      <c r="H6" s="21"/>
-    </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G6" s="21" t="s">
+        <v>905</v>
+      </c>
+      <c r="H6" t="s">
+        <v>917</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
         <v>266</v>
       </c>
@@ -12756,12 +12857,16 @@
         <v>2</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G7" s="16"/>
-      <c r="H7" s="16"/>
-    </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>906</v>
+      </c>
+      <c r="H7" s="16" t="s">
+        <v>917</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="19" t="s">
         <v>266</v>
       </c>
@@ -12778,12 +12883,14 @@
         <v>3</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G8" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G8" s="21" t="s">
+        <v>907</v>
+      </c>
       <c r="H8" s="21"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
         <v>266</v>
       </c>
@@ -12800,12 +12907,16 @@
         <v>3</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G9" s="16"/>
-      <c r="H9" s="16"/>
-    </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G9" s="16" t="s">
+        <v>908</v>
+      </c>
+      <c r="H9" s="16" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="19" t="s">
         <v>266</v>
       </c>
@@ -12822,12 +12933,16 @@
         <v>3</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G10" s="21"/>
-      <c r="H10" s="21"/>
-    </row>
-    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G10" s="21" t="s">
+        <v>909</v>
+      </c>
+      <c r="H10" s="21" t="s">
+        <v>921</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
         <v>280</v>
       </c>
@@ -12841,7 +12956,7 @@
       <c r="G11" s="13"/>
       <c r="H11" s="13"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>280</v>
       </c>
@@ -12858,12 +12973,14 @@
         <v>1</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G12" s="16"/>
+        <v>916</v>
+      </c>
+      <c r="G12" s="16" t="s">
+        <v>910</v>
+      </c>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="19" t="s">
         <v>280</v>
       </c>
@@ -12880,12 +12997,14 @@
         <v>1</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G13" s="21"/>
+        <v>916</v>
+      </c>
+      <c r="G13" s="21" t="s">
+        <v>911</v>
+      </c>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="14" t="s">
         <v>280</v>
       </c>
@@ -12902,12 +13021,16 @@
         <v>3</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G14" s="16"/>
-      <c r="H14" s="16"/>
-    </row>
-    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G14" s="16" t="s">
+        <v>912</v>
+      </c>
+      <c r="H14" s="16" t="s">
+        <v>920</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="13" t="s">
         <v>288</v>
       </c>
@@ -12921,7 +13044,7 @@
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="14" t="s">
         <v>288</v>
       </c>
@@ -12938,12 +13061,16 @@
         <v>2</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G16" s="16"/>
-      <c r="H16" s="16"/>
-    </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G16" s="16" t="s">
+        <v>913</v>
+      </c>
+      <c r="H16" s="16" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="19" t="s">
         <v>288</v>
       </c>
@@ -12960,12 +13087,16 @@
         <v>2</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G17" s="21"/>
-      <c r="H17" s="21"/>
-    </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G17" s="21" t="s">
+        <v>914</v>
+      </c>
+      <c r="H17" t="s">
+        <v>918</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="14" t="s">
         <v>288</v>
       </c>
@@ -12982,10 +13113,14 @@
         <v>2</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G18" s="16"/>
-      <c r="H18" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G18" s="16" t="s">
+        <v>915</v>
+      </c>
+      <c r="H18" s="16" t="s">
+        <v>922</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F18">
@@ -13013,7 +13148,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:H56"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -13025,7 +13160,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -13051,7 +13186,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>296</v>
       </c>
@@ -13065,7 +13200,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>296</v>
       </c>
@@ -13087,7 +13222,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>296</v>
       </c>
@@ -13109,7 +13244,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>296</v>
       </c>
@@ -13131,7 +13266,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="13" t="s">
         <v>304</v>
       </c>
@@ -13145,7 +13280,7 @@
       <c r="G6" s="13"/>
       <c r="H6" s="13"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
         <v>304</v>
       </c>
@@ -13167,7 +13302,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="19" t="s">
         <v>304</v>
       </c>
@@ -13189,7 +13324,7 @@
       <c r="G8" s="21"/>
       <c r="H8" s="21"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
         <v>304</v>
       </c>
@@ -13211,7 +13346,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="19" t="s">
         <v>304</v>
       </c>
@@ -13233,7 +13368,7 @@
       <c r="G10" s="21"/>
       <c r="H10" s="21"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="14" t="s">
         <v>304</v>
       </c>
@@ -13255,7 +13390,7 @@
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="19" t="s">
         <v>304</v>
       </c>
@@ -13277,7 +13412,7 @@
       <c r="G12" s="21"/>
       <c r="H12" s="21"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
         <v>304</v>
       </c>
@@ -13299,7 +13434,7 @@
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="19" t="s">
         <v>304</v>
       </c>
@@ -13321,7 +13456,7 @@
       <c r="G14" s="21"/>
       <c r="H14" s="21"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
         <v>304</v>
       </c>
@@ -13343,7 +13478,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>304</v>
       </c>
@@ -13365,7 +13500,7 @@
       <c r="G16" s="21"/>
       <c r="H16" s="21"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="14" t="s">
         <v>304</v>
       </c>
@@ -13387,7 +13522,7 @@
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="19" t="s">
         <v>304</v>
       </c>
@@ -13409,7 +13544,7 @@
       <c r="G18" s="21"/>
       <c r="H18" s="21"/>
     </row>
-    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="13" t="s">
         <v>330</v>
       </c>
@@ -13423,7 +13558,7 @@
       <c r="G19" s="13"/>
       <c r="H19" s="13"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="14" t="s">
         <v>330</v>
       </c>
@@ -13445,7 +13580,7 @@
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="19" t="s">
         <v>330</v>
       </c>
@@ -13467,7 +13602,7 @@
       <c r="G21" s="21"/>
       <c r="H21" s="21"/>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="14" t="s">
         <v>330</v>
       </c>
@@ -13489,7 +13624,7 @@
       <c r="G22" s="16"/>
       <c r="H22" s="16"/>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="19" t="s">
         <v>330</v>
       </c>
@@ -13511,7 +13646,7 @@
       <c r="G23" s="21"/>
       <c r="H23" s="21"/>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="14" t="s">
         <v>330</v>
       </c>
@@ -13533,7 +13668,7 @@
       <c r="G24" s="16"/>
       <c r="H24" s="16"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="19" t="s">
         <v>330</v>
       </c>
@@ -13555,7 +13690,7 @@
       <c r="G25" s="21"/>
       <c r="H25" s="21"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="14" t="s">
         <v>330</v>
       </c>
@@ -13577,7 +13712,7 @@
       <c r="G26" s="16"/>
       <c r="H26" s="16"/>
     </row>
-    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="19" t="s">
         <v>330</v>
       </c>
@@ -13599,7 +13734,7 @@
       <c r="G27" s="21"/>
       <c r="H27" s="21"/>
     </row>
-    <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="13" t="s">
         <v>348</v>
       </c>
@@ -13613,7 +13748,7 @@
       <c r="G28" s="13"/>
       <c r="H28" s="13"/>
     </row>
-    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="14" t="s">
         <v>348</v>
       </c>
@@ -13635,7 +13770,7 @@
       <c r="G29" s="16"/>
       <c r="H29" s="16"/>
     </row>
-    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="19" t="s">
         <v>348</v>
       </c>
@@ -13657,7 +13792,7 @@
       <c r="G30" s="21"/>
       <c r="H30" s="21"/>
     </row>
-    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="14" t="s">
         <v>348</v>
       </c>
@@ -13679,7 +13814,7 @@
       <c r="G31" s="16"/>
       <c r="H31" s="16"/>
     </row>
-    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="19" t="s">
         <v>348</v>
       </c>
@@ -13701,7 +13836,7 @@
       <c r="G32" s="21"/>
       <c r="H32" s="21"/>
     </row>
-    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="14" t="s">
         <v>348</v>
       </c>
@@ -13723,7 +13858,7 @@
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
     </row>
-    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="19" t="s">
         <v>348</v>
       </c>
@@ -13745,7 +13880,7 @@
       <c r="G34" s="21"/>
       <c r="H34" s="21"/>
     </row>
-    <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="13" t="s">
         <v>362</v>
       </c>
@@ -13759,7 +13894,7 @@
       <c r="G35" s="13"/>
       <c r="H35" s="13"/>
     </row>
-    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="14" t="s">
         <v>362</v>
       </c>
@@ -13781,7 +13916,7 @@
       <c r="G36" s="16"/>
       <c r="H36" s="16"/>
     </row>
-    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="19" t="s">
         <v>362</v>
       </c>
@@ -13803,7 +13938,7 @@
       <c r="G37" s="21"/>
       <c r="H37" s="21"/>
     </row>
-    <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="14" t="s">
         <v>362</v>
       </c>
@@ -13825,7 +13960,7 @@
       <c r="G38" s="16"/>
       <c r="H38" s="16"/>
     </row>
-    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="19" t="s">
         <v>362</v>
       </c>
@@ -13847,7 +13982,7 @@
       <c r="G39" s="21"/>
       <c r="H39" s="21"/>
     </row>
-    <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="14" t="s">
         <v>362</v>
       </c>
@@ -13869,7 +14004,7 @@
       <c r="G40" s="16"/>
       <c r="H40" s="16"/>
     </row>
-    <row r="41" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="19" t="s">
         <v>362</v>
       </c>
@@ -13891,7 +14026,7 @@
       <c r="G41" s="21"/>
       <c r="H41" s="21"/>
     </row>
-    <row r="42" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="14" t="s">
         <v>362</v>
       </c>
@@ -13913,7 +14048,7 @@
       <c r="G42" s="16"/>
       <c r="H42" s="16"/>
     </row>
-    <row r="43" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="19" t="s">
         <v>362</v>
       </c>
@@ -13935,7 +14070,7 @@
       <c r="G43" s="21"/>
       <c r="H43" s="21"/>
     </row>
-    <row r="44" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="13" t="s">
         <v>380</v>
       </c>
@@ -13949,7 +14084,7 @@
       <c r="G44" s="13"/>
       <c r="H44" s="13"/>
     </row>
-    <row r="45" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="14" t="s">
         <v>380</v>
       </c>
@@ -13971,7 +14106,7 @@
       <c r="G45" s="16"/>
       <c r="H45" s="16"/>
     </row>
-    <row r="46" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="19" t="s">
         <v>380</v>
       </c>
@@ -13993,7 +14128,7 @@
       <c r="G46" s="21"/>
       <c r="H46" s="21"/>
     </row>
-    <row r="47" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="14" t="s">
         <v>380</v>
       </c>
@@ -14015,7 +14150,7 @@
       <c r="G47" s="16"/>
       <c r="H47" s="16"/>
     </row>
-    <row r="48" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="19" t="s">
         <v>380</v>
       </c>
@@ -14037,7 +14172,7 @@
       <c r="G48" s="21"/>
       <c r="H48" s="21"/>
     </row>
-    <row r="49" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="13" t="s">
         <v>390</v>
       </c>
@@ -14051,7 +14186,7 @@
       <c r="G49" s="13"/>
       <c r="H49" s="13"/>
     </row>
-    <row r="50" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="14" t="s">
         <v>390</v>
       </c>
@@ -14073,7 +14208,7 @@
       <c r="G50" s="16"/>
       <c r="H50" s="16"/>
     </row>
-    <row r="51" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="19" t="s">
         <v>390</v>
       </c>
@@ -14095,7 +14230,7 @@
       <c r="G51" s="21"/>
       <c r="H51" s="21"/>
     </row>
-    <row r="52" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="13" t="s">
         <v>396</v>
       </c>
@@ -14109,7 +14244,7 @@
       <c r="G52" s="13"/>
       <c r="H52" s="13"/>
     </row>
-    <row r="53" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="14" t="s">
         <v>396</v>
       </c>
@@ -14131,7 +14266,7 @@
       <c r="G53" s="16"/>
       <c r="H53" s="16"/>
     </row>
-    <row r="54" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="19" t="s">
         <v>396</v>
       </c>
@@ -14153,7 +14288,7 @@
       <c r="G54" s="21"/>
       <c r="H54" s="21"/>
     </row>
-    <row r="55" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="14" t="s">
         <v>396</v>
       </c>
@@ -14175,7 +14310,7 @@
       <c r="G55" s="16"/>
       <c r="H55" s="16"/>
     </row>
-    <row r="56" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="19" t="s">
         <v>396</v>
       </c>
@@ -14223,7 +14358,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:H26"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -14235,7 +14370,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -14261,7 +14396,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>406</v>
       </c>
@@ -14275,7 +14410,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>406</v>
       </c>
@@ -14296,10 +14431,10 @@
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="16" t="s">
-        <v>902</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>899</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>406</v>
       </c>
@@ -14320,10 +14455,10 @@
       </c>
       <c r="G4" s="21"/>
       <c r="H4" s="21" t="s">
-        <v>903</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>406</v>
       </c>
@@ -14345,7 +14480,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="13" t="s">
         <v>414</v>
       </c>
@@ -14359,7 +14494,7 @@
       <c r="G6" s="13"/>
       <c r="H6" s="13"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
         <v>414</v>
       </c>
@@ -14381,7 +14516,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="19" t="s">
         <v>414</v>
       </c>
@@ -14403,7 +14538,7 @@
       <c r="G8" s="21"/>
       <c r="H8" s="21"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
         <v>414</v>
       </c>
@@ -14425,7 +14560,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="19" t="s">
         <v>414</v>
       </c>
@@ -14447,7 +14582,7 @@
       <c r="G10" s="21"/>
       <c r="H10" s="21"/>
     </row>
-    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
         <v>424</v>
       </c>
@@ -14461,7 +14596,7 @@
       <c r="G11" s="13"/>
       <c r="H11" s="13"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>424</v>
       </c>
@@ -14483,7 +14618,7 @@
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="19" t="s">
         <v>424</v>
       </c>
@@ -14505,7 +14640,7 @@
       <c r="G13" s="21"/>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="13" t="s">
         <v>430</v>
       </c>
@@ -14519,7 +14654,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
         <v>430</v>
       </c>
@@ -14541,7 +14676,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>430</v>
       </c>
@@ -14563,7 +14698,7 @@
       <c r="G16" s="21"/>
       <c r="H16" s="21"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="14" t="s">
         <v>430</v>
       </c>
@@ -14585,7 +14720,7 @@
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="19" t="s">
         <v>430</v>
       </c>
@@ -14607,7 +14742,7 @@
       <c r="G18" s="21"/>
       <c r="H18" s="21"/>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="14" t="s">
         <v>430</v>
       </c>
@@ -14629,7 +14764,7 @@
       <c r="G19" s="16"/>
       <c r="H19" s="16"/>
     </row>
-    <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="13" t="s">
         <v>442</v>
       </c>
@@ -14643,7 +14778,7 @@
       <c r="G20" s="13"/>
       <c r="H20" s="13"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="14" t="s">
         <v>442</v>
       </c>
@@ -14665,7 +14800,7 @@
       <c r="G21" s="16"/>
       <c r="H21" s="16"/>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="19" t="s">
         <v>442</v>
       </c>
@@ -14687,7 +14822,7 @@
       <c r="G22" s="21"/>
       <c r="H22" s="21"/>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="14" t="s">
         <v>442</v>
       </c>
@@ -14709,7 +14844,7 @@
       <c r="G23" s="16"/>
       <c r="H23" s="16"/>
     </row>
-    <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="13" t="s">
         <v>450</v>
       </c>
@@ -14723,7 +14858,7 @@
       <c r="G24" s="13"/>
       <c r="H24" s="13"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="14" t="s">
         <v>450</v>
       </c>
@@ -14745,7 +14880,7 @@
       <c r="G25" s="16"/>
       <c r="H25" s="16"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="19" t="s">
         <v>450</v>
       </c>
@@ -14793,7 +14928,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -14805,7 +14940,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -14831,7 +14966,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>456</v>
       </c>
@@ -14845,7 +14980,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>456</v>
       </c>
@@ -14865,13 +15000,13 @@
         <v>892</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="H3" s="16" t="s">
-        <v>897</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>924</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>456</v>
       </c>
@@ -14888,16 +15023,16 @@
         <v>2</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G4" s="21" t="s">
-        <v>899</v>
+        <v>892</v>
+      </c>
+      <c r="G4" s="27" t="s">
+        <v>926</v>
       </c>
       <c r="H4" s="21" t="s">
-        <v>900</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>925</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>456</v>
       </c>
@@ -14919,7 +15054,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>456</v>
       </c>
@@ -14936,12 +15071,14 @@
         <v>3</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G6" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G6" s="21" t="s">
+        <v>923</v>
+      </c>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="13" t="s">
         <v>466</v>
       </c>
@@ -14955,7 +15092,7 @@
       <c r="G7" s="13"/>
       <c r="H7" s="13"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="14" t="s">
         <v>466</v>
       </c>
@@ -14972,12 +15109,16 @@
         <v>1</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
-    </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G8" s="16" t="s">
+        <v>928</v>
+      </c>
+      <c r="H8" s="16" t="s">
+        <v>929</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="19" t="s">
         <v>466</v>
       </c>
@@ -14994,12 +15135,16 @@
         <v>1</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G9" s="21"/>
-      <c r="H9" s="21"/>
-    </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G9" s="21" t="s">
+        <v>927</v>
+      </c>
+      <c r="H9" s="21" t="s">
+        <v>930</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="14" t="s">
         <v>466</v>
       </c>
@@ -15021,7 +15166,7 @@
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="19" t="s">
         <v>466</v>
       </c>
@@ -15038,12 +15183,12 @@
         <v>3</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>45</v>
+        <v>892</v>
       </c>
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="13" t="s">
         <v>476</v>
       </c>
@@ -15057,7 +15202,7 @@
       <c r="G12" s="13"/>
       <c r="H12" s="13"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
         <v>476</v>
       </c>
@@ -15074,12 +15219,16 @@
         <v>1</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G13" s="16"/>
-      <c r="H13" s="16"/>
-    </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G13" s="16" t="s">
+        <v>931</v>
+      </c>
+      <c r="H13" s="16" t="s">
+        <v>932</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="19" t="s">
         <v>476</v>
       </c>
@@ -15101,7 +15250,7 @@
       <c r="G14" s="21"/>
       <c r="H14" s="21"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
         <v>476</v>
       </c>
@@ -15118,12 +15267,16 @@
         <v>3</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G15" s="16"/>
-      <c r="H15" s="16"/>
-    </row>
-    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G15" s="16" t="s">
+        <v>933</v>
+      </c>
+      <c r="H15" s="16" t="s">
+        <v>930</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="13" t="s">
         <v>484</v>
       </c>
@@ -15137,7 +15290,7 @@
       <c r="G16" s="13"/>
       <c r="H16" s="13"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="14" t="s">
         <v>484</v>
       </c>
@@ -15154,12 +15307,12 @@
         <v>2</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>45</v>
+        <v>894</v>
       </c>
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="19" t="s">
         <v>484</v>
       </c>
@@ -15176,10 +15329,14 @@
         <v>3</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G18" s="21"/>
-      <c r="H18" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G18" s="21" t="s">
+        <v>934</v>
+      </c>
+      <c r="H18" s="21" t="s">
+        <v>935</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F18">

</xml_diff>

<commit_message>
docs(asvs): align input validation and sanitization controls with chat and file modules
</commit_message>
<xml_diff>
--- a/Deliverables/Phase1/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/Phase1/ASVS_5.0_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ambiente de Trabalho\2º semestre\DESOFT\desofs2026-wed_nap_5\Deliverables\Phase1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FFD66DE-621F-4BDB-864C-9D42EBD2FA94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69EC001A-08F7-49CC-9E86-9BA0CC5E92AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" firstSheet="8" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2103" uniqueCount="936">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2119" uniqueCount="945">
   <si>
     <t>OWASP ASVS 5.0 – Compliance Tracker</t>
   </si>
@@ -2873,6 +2873,33 @@
   </si>
   <si>
     <t>SR2, SR4, SR16</t>
+  </si>
+  <si>
+    <t>Output encoding and sanitization are applied to user-generated content, particularly in chat messages, to prevent XSS attacks.</t>
+  </si>
+  <si>
+    <t>SR10, AC8</t>
+  </si>
+  <si>
+    <t>Output encoding is considered for responses to prevent injection vulnerabilities such as XSS.</t>
+  </si>
+  <si>
+    <t>Database interactions are protected using safe query mechanisms and input validation to prevent SQL injection.</t>
+  </si>
+  <si>
+    <t>Input validation reduces the risk of command injection by restricting untrusted input.</t>
+  </si>
+  <si>
+    <t>Input validation and sanitization mechanisms are applied to prevent injection through special characters.</t>
+  </si>
+  <si>
+    <t>User-generated content (chat messages) is sanitized to prevent execution of malicious scripts such as XSS.</t>
+  </si>
+  <si>
+    <t>Input data is validated and sanitized before being used in sensitive contexts.</t>
+  </si>
+  <si>
+    <t>Untrusted input is sanitized before being stored or processed to prevent injection attacks.</t>
   </si>
 </sst>
 </file>
@@ -3030,7 +3057,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3102,9 +3129,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10269,10 +10293,14 @@
         <v>2</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G4" s="21" t="s">
+        <v>936</v>
+      </c>
+      <c r="H4" s="21" t="s">
+        <v>937</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="13" t="s">
@@ -10305,10 +10333,14 @@
         <v>1</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G6" s="16" t="s">
+        <v>938</v>
+      </c>
+      <c r="H6" s="16" t="s">
+        <v>918</v>
+      </c>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="19" t="s">
@@ -10371,10 +10403,14 @@
         <v>1</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G9" s="21"/>
-      <c r="H9" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G9" s="21" t="s">
+        <v>939</v>
+      </c>
+      <c r="H9" s="21" t="s">
+        <v>918</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="14" t="s">
@@ -10393,10 +10429,14 @@
         <v>1</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G10" s="16"/>
-      <c r="H10" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G10" s="16" t="s">
+        <v>940</v>
+      </c>
+      <c r="H10" s="16" t="s">
+        <v>918</v>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="19" t="s">
@@ -10481,10 +10521,14 @@
         <v>2</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G14" s="16"/>
-      <c r="H14" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G14" s="16" t="s">
+        <v>941</v>
+      </c>
+      <c r="H14" s="16" t="s">
+        <v>918</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="19" t="s">
@@ -10539,10 +10583,14 @@
         <v>1</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G17" s="16"/>
-      <c r="H17" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G17" s="16" t="s">
+        <v>942</v>
+      </c>
+      <c r="H17" s="16" t="s">
+        <v>937</v>
+      </c>
     </row>
     <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="19" t="s">
@@ -10583,10 +10631,14 @@
         <v>2</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G19" s="16"/>
-      <c r="H19" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G19" s="16" t="s">
+        <v>943</v>
+      </c>
+      <c r="H19" s="16" t="s">
+        <v>918</v>
+      </c>
     </row>
     <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="19" t="s">
@@ -10715,10 +10767,14 @@
         <v>2</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G25" s="16"/>
-      <c r="H25" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G25" s="16" t="s">
+        <v>944</v>
+      </c>
+      <c r="H25" s="16" t="s">
+        <v>918</v>
+      </c>
     </row>
     <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="19" t="s">
@@ -15025,7 +15081,7 @@
       <c r="F4" s="18" t="s">
         <v>892</v>
       </c>
-      <c r="G4" s="27" t="s">
+      <c r="G4" s="21" t="s">
         <v>926</v>
       </c>
       <c r="H4" s="21" t="s">

</xml_diff>

<commit_message>
docs(asvs): align TLS and HTTPS communication controls with security architecture
</commit_message>
<xml_diff>
--- a/Deliverables/Phase1/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/Phase1/ASVS_5.0_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ambiente de Trabalho\2º semestre\DESOFT\desofs2026-wed_nap_5\Deliverables\Phase1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69EC001A-08F7-49CC-9E86-9BA0CC5E92AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A686CDC-51F9-47F2-89EE-08FB1EB51C5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" firstSheet="11" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2119" uniqueCount="945">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2129" uniqueCount="951">
   <si>
     <t>OWASP ASVS 5.0 – Compliance Tracker</t>
   </si>
@@ -2900,6 +2900,24 @@
   </si>
   <si>
     <t>Untrusted input is sanitized before being stored or processed to prevent injection attacks.</t>
+  </si>
+  <si>
+    <t>The system enforces secure communication using TLS 1.3 for all external connections.</t>
+  </si>
+  <si>
+    <t>SR13</t>
+  </si>
+  <si>
+    <t>All communication between clients and the system is enforced over HTTPS, with no fallback to insecure protocols.</t>
+  </si>
+  <si>
+    <t>External services are expected to use trusted TLS certificates for secure communication.</t>
+  </si>
+  <si>
+    <t>Secure communication using TLS is enforced for internal and external data flows within the system.</t>
+  </si>
+  <si>
+    <t>Transport layer encryption is applied to internal service communication to ensure confidentiality and integrity.</t>
   </si>
 </sst>
 </file>
@@ -3386,7 +3404,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0</c:v>
+                  <c:v>0.33333333333333331</c:v>
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>0</c:v>
@@ -3935,7 +3953,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0</c:v>
+                  <c:v>8.3333333333333329E-2</c:v>
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>0</c:v>
@@ -5108,11 +5126,11 @@
       </c>
       <c r="D17" s="7">
         <f>COUNTIFS('V12 - Secure Communication'!$F$2:$F$16,"Compliant",'V12 - Secure Communication'!$E$2:$E$16,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E17" s="8">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="F17" s="7">
         <v>6</v>
@@ -5138,11 +5156,11 @@
       </c>
       <c r="L17" s="7">
         <f>COUNTIF('V12 - Secure Communication'!$F$2:$F$16,"Compliant")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M17" s="8">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>8.3333333333333329E-2</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
@@ -5400,11 +5418,11 @@
       </c>
       <c r="D23" s="10">
         <f>SUM(D6:D22)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E23" s="11">
         <f>IFERROR(AVERAGE(E6:E22),"")</f>
-        <v>3.3333333333333333E-2</v>
+        <v>5.5555555555555552E-2</v>
       </c>
       <c r="F23" s="10">
         <f>SUM(F6:F22)</f>
@@ -5432,11 +5450,11 @@
       </c>
       <c r="L23" s="10">
         <f>SUM(L6:L22)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M23" s="11">
         <f>IFERROR(AVERAGE(M6:M22),"")</f>
-        <v>1.3574660633484163E-2</v>
+        <v>1.8476621417797889E-2</v>
       </c>
     </row>
   </sheetData>
@@ -7461,10 +7479,14 @@
         <v>1</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>945</v>
+      </c>
+      <c r="H3" s="16" t="s">
+        <v>946</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
@@ -7585,10 +7607,14 @@
         <v>1</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G9" s="16"/>
-      <c r="H9" s="16"/>
+        <v>916</v>
+      </c>
+      <c r="G9" s="16" t="s">
+        <v>947</v>
+      </c>
+      <c r="H9" s="16" t="s">
+        <v>946</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="19" t="s">
@@ -7607,10 +7633,14 @@
         <v>1</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G10" s="21"/>
-      <c r="H10" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G10" s="21" t="s">
+        <v>948</v>
+      </c>
+      <c r="H10" s="21" t="s">
+        <v>946</v>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
@@ -7643,10 +7673,14 @@
         <v>2</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G12" s="16"/>
-      <c r="H12" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G12" s="16" t="s">
+        <v>949</v>
+      </c>
+      <c r="H12" s="16" t="s">
+        <v>946</v>
+      </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="19" t="s">
@@ -7687,10 +7721,14 @@
         <v>2</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G14" s="16"/>
-      <c r="H14" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G14" s="16" t="s">
+        <v>950</v>
+      </c>
+      <c r="H14" s="16" t="s">
+        <v>946</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="19" t="s">

</xml_diff>

<commit_message>
docs(asvs): align logging and monitoring controls with security requirements
</commit_message>
<xml_diff>
--- a/Deliverables/Phase1/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/Phase1/ASVS_5.0_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ambiente de Trabalho\2º semestre\DESOFT\desofs2026-wed_nap_5\Deliverables\Phase1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A686CDC-51F9-47F2-89EE-08FB1EB51C5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E86A677-3658-4071-977C-EC5B16D6C57A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" firstSheet="11" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" firstSheet="15" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2129" uniqueCount="951">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2155" uniqueCount="972">
   <si>
     <t>OWASP ASVS 5.0 – Compliance Tracker</t>
   </si>
@@ -2918,13 +2918,76 @@
   </si>
   <si>
     <t>Transport layer encryption is applied to internal service communication to ensure confidentiality and integrity.</t>
+  </si>
+  <si>
+    <t>Logging requirements and events are defined, including authentication and critical system actions.</t>
+  </si>
+  <si>
+    <t>FR23-27, SR16</t>
+  </si>
+  <si>
+    <t>Logs include metadata such as timestamp, user identifier, and action details.</t>
+  </si>
+  <si>
+    <t>FR25, FR26, FR27</t>
+  </si>
+  <si>
+    <t>Timestamps are included in logs, although time synchronization details are not fully specified.</t>
+  </si>
+  <si>
+    <t>FR25</t>
+  </si>
+  <si>
+    <t>Logs are structured to support monitoring and analysis of system activity.</t>
+  </si>
+  <si>
+    <t>SR16</t>
+  </si>
+  <si>
+    <t>Sensitive data is excluded from logs according to security requirements.</t>
+  </si>
+  <si>
+    <t>SR17</t>
+  </si>
+  <si>
+    <t>Authentication events, including login attempts, are logged.</t>
+  </si>
+  <si>
+    <t>FR23, SR16</t>
+  </si>
+  <si>
+    <t>Authorization and access control failures are considered for logging.</t>
+  </si>
+  <si>
+    <t>Security-relevant events and suspicious actions are logged for monitoring.</t>
+  </si>
+  <si>
+    <t>System errors and failures are logged to support debugging and incident response.</t>
+  </si>
+  <si>
+    <t>FR24, SR16</t>
+  </si>
+  <si>
+    <t>Input validation reduces the risk of log injection attacks.</t>
+  </si>
+  <si>
+    <t>Logs are expected to be protected from unauthorized access through system-level controls.</t>
+  </si>
+  <si>
+    <t>Error handling mechanisms avoid exposing sensitive information to users.</t>
+  </si>
+  <si>
+    <t>The system is designed to handle failures without compromising security.</t>
+  </si>
+  <si>
+    <t>NFR5</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -2989,6 +3052,12 @@
       <sz val="10"/>
       <color rgb="FF1F3864"/>
       <name val="Cambria"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -3600,7 +3669,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0</c:v>
+                  <c:v>0.125</c:v>
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>0</c:v>
@@ -3965,7 +4034,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0</c:v>
+                  <c:v>0.11764705882352941</c:v>
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>0</c:v>
@@ -5331,11 +5400,11 @@
       </c>
       <c r="G21" s="7">
         <f>COUNTIFS('V16 - Security Logging and Erro'!$F$2:$F$23,"Compliant",'V16 - Security Logging and Erro'!$E$2:$E$23,2)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H21" s="8">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I21" s="7">
         <v>1</v>
@@ -5350,11 +5419,11 @@
       </c>
       <c r="L21" s="7">
         <f>COUNTIF('V16 - Security Logging and Erro'!$F$2:$F$23,"Compliant")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M21" s="8">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.11764705882352941</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
@@ -5430,11 +5499,11 @@
       </c>
       <c r="G23" s="10">
         <f>SUM(G6:G22)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H23" s="11">
         <f>IFERROR(AVERAGE(H6:H22),"")</f>
-        <v>1.1764705882352941E-2</v>
+        <v>1.9117647058823531E-2</v>
       </c>
       <c r="I23" s="10">
         <f>SUM(I6:I22)</f>
@@ -5450,11 +5519,11 @@
       </c>
       <c r="L23" s="10">
         <f>SUM(L6:L22)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M23" s="11">
         <f>IFERROR(AVERAGE(M6:M22),"")</f>
-        <v>1.8476621417797889E-2</v>
+        <v>2.5397036642711385E-2</v>
       </c>
     </row>
   </sheetData>
@@ -9431,10 +9500,14 @@
         <v>2</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>951</v>
+      </c>
+      <c r="H3" s="16" t="s">
+        <v>952</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="13" t="s">
@@ -9467,10 +9540,14 @@
         <v>2</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
+        <v>916</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>953</v>
+      </c>
+      <c r="H5" s="16" t="s">
+        <v>954</v>
+      </c>
     </row>
     <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
@@ -9489,10 +9566,14 @@
         <v>2</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G6" s="21"/>
-      <c r="H6" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G6" s="21" t="s">
+        <v>955</v>
+      </c>
+      <c r="H6" s="21" t="s">
+        <v>956</v>
+      </c>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
@@ -9533,10 +9614,14 @@
         <v>2</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G8" s="21"/>
-      <c r="H8" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G8" s="21" t="s">
+        <v>957</v>
+      </c>
+      <c r="H8" s="21" t="s">
+        <v>958</v>
+      </c>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
@@ -9555,10 +9640,14 @@
         <v>2</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G9" s="16"/>
-      <c r="H9" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G9" s="16" t="s">
+        <v>959</v>
+      </c>
+      <c r="H9" s="16" t="s">
+        <v>960</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="13" t="s">
@@ -9591,10 +9680,14 @@
         <v>2</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G11" s="16"/>
-      <c r="H11" s="16"/>
+        <v>916</v>
+      </c>
+      <c r="G11" s="16" t="s">
+        <v>961</v>
+      </c>
+      <c r="H11" s="16" t="s">
+        <v>962</v>
+      </c>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="19" t="s">
@@ -9613,10 +9706,14 @@
         <v>2</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G12" s="21"/>
-      <c r="H12" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G12" s="21" t="s">
+        <v>963</v>
+      </c>
+      <c r="H12" s="21" t="s">
+        <v>958</v>
+      </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
@@ -9635,10 +9732,14 @@
         <v>2</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G13" s="16"/>
-      <c r="H13" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G13" s="16" t="s">
+        <v>964</v>
+      </c>
+      <c r="H13" s="21" t="s">
+        <v>958</v>
+      </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="19" t="s">
@@ -9657,10 +9758,14 @@
         <v>2</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G14" s="21"/>
-      <c r="H14" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G14" s="21" t="s">
+        <v>965</v>
+      </c>
+      <c r="H14" s="21" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="13" t="s">
@@ -9693,10 +9798,14 @@
         <v>2</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G16" s="16"/>
-      <c r="H16" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G16" s="16" t="s">
+        <v>967</v>
+      </c>
+      <c r="H16" s="16" t="s">
+        <v>918</v>
+      </c>
     </row>
     <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="19" t="s">
@@ -9715,10 +9824,14 @@
         <v>2</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G17" s="21"/>
-      <c r="H17" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G17" s="21" t="s">
+        <v>968</v>
+      </c>
+      <c r="H17" s="21" t="s">
+        <v>958</v>
+      </c>
     </row>
     <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="14" t="s">
@@ -9773,10 +9886,14 @@
         <v>2</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G20" s="16"/>
-      <c r="H20" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G20" s="16" t="s">
+        <v>969</v>
+      </c>
+      <c r="H20" s="16" t="s">
+        <v>960</v>
+      </c>
     </row>
     <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="19" t="s">
@@ -9797,8 +9914,6 @@
       <c r="F21" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="G21" s="21"/>
-      <c r="H21" s="21"/>
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="14" t="s">
@@ -9817,10 +9932,14 @@
         <v>2</v>
       </c>
       <c r="F22" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G22" s="16"/>
-      <c r="H22" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G22" s="21" t="s">
+        <v>970</v>
+      </c>
+      <c r="H22" s="21" t="s">
+        <v>971</v>
+      </c>
     </row>
     <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="19" t="s">
@@ -9845,6 +9964,7 @@
       <c r="H23" s="21"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="10" type="noConversion"/>
   <conditionalFormatting sqref="F2:F23">
     <cfRule type="cellIs" priority="2" operator="equal">
       <formula>"Compliant"</formula>

</xml_diff>

<commit_message>
Improve ASVS V1 and V2 tracker mappings and observations
</commit_message>
<xml_diff>
--- a/Deliverables/Phase1/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/Phase1/ASVS_5.0_Tracker.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabio\Documents\isep\DESOFS\desofs2026-wed_nap_5\Deliverables\Phase1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ambiente de Trabalho\2º semestre\DESOFT\desofs2026-wed_nap_5\Deliverables\Phase1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D6241DD-95FF-4A2C-A1F2-F84F0592F38D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC0DF09E-26C8-4293-B52A-37FC33125C09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="13" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2155" uniqueCount="972">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2191" uniqueCount="997">
   <si>
     <t>OWASP ASVS 5.0 – Compliance Tracker</t>
   </si>
@@ -2981,6 +2981,81 @@
   </si>
   <si>
     <t>NFR5</t>
+  </si>
+  <si>
+    <t>Dynamic URLs and query parameters are validated and encoded to reduce injection risks through manipulated input.</t>
+  </si>
+  <si>
+    <t>Dynamic content included in JSON responses is encoded and validated before being processed by the client.</t>
+  </si>
+  <si>
+    <t>Unsafe dynamic code execution mechanisms such as eval or unrestricted expression parsing are avoided.</t>
+  </si>
+  <si>
+    <t>User-generated content is sanitized before rendering to prevent template and script injection attacks.</t>
+  </si>
+  <si>
+    <t>Untrusted serialized input is validated and processed using safe deserialization mechanisms.</t>
+  </si>
+  <si>
+    <t>The application is implemented using Java, a managed memory-safe language that reduces risks related to unsafe memory operations.</t>
+  </si>
+  <si>
+    <t>NFR9</t>
+  </si>
+  <si>
+    <t>Built-in language protections and input validation reduce risks related to integer handling and unsafe memory operations.</t>
+  </si>
+  <si>
+    <t>Memory management and resource cleanup are automatically handled by the JVM and garbage collector.</t>
+  </si>
+  <si>
+    <t>Business rules and contextual validations are documented for authentication, enrollment, file access, and chat authorization flows.</t>
+  </si>
+  <si>
+    <t>SR4, SR5, SR6</t>
+  </si>
+  <si>
+    <t>Business logic limits and validation rules are defined for uploads, authentication attempts, and course access operations.</t>
+  </si>
+  <si>
+    <t>NFR5, SR3, SR11</t>
+  </si>
+  <si>
+    <t>User input is validated using predefined rules, expected formats, and server-side validation mechanisms.</t>
+  </si>
+  <si>
+    <t>Input validation is enforced at the backend service layer and is not dependent on client-side validation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SR10 </t>
+  </si>
+  <si>
+    <t>Related data validation rules are applied to ensure logical consistency between users, enrollments, and course resources.</t>
+  </si>
+  <si>
+    <t>Business workflows enforce sequential processing and authorization checks before sensitive operations are executed.</t>
+  </si>
+  <si>
+    <t>Business logic restrictions are applied to uploads, enrollments, and access-control operations to reduce abuse scenarios.</t>
+  </si>
+  <si>
+    <t>SR5, SR11</t>
+  </si>
+  <si>
+    <t>Transactional operations are handled consistently to preserve application state integrity during critical operations.</t>
+  </si>
+  <si>
+    <t>NFR4</t>
+  </si>
+  <si>
+    <t>Rate limiting and validation controls are planned to reduce abuse of authentication and upload operations.</t>
+  </si>
+  <si>
+    <t>SR3</t>
+  </si>
+  <si>
+    <t>Sensitive code changes require peer review and merge request approval before integration into protected branches.</t>
   </si>
 </sst>
 </file>
@@ -3304,7 +3379,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="pt-BR"/>
+  <c:lang val="pt-PT"/>
   <c:roundedCorners val="0"/>
   <c:style val="2"/>
   <c:chart>
@@ -3624,7 +3699,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="17"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>0.15789473684210525</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -3989,7 +4064,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="17"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -4550,13 +4625,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P23"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
     <col min="2" max="13" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
@@ -4576,7 +4651,7 @@
       <c r="O1" s="24"/>
       <c r="P1" s="24"/>
     </row>
-    <row r="2" spans="1:16" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="25"/>
       <c r="B2" s="25"/>
       <c r="C2" s="25"/>
@@ -4594,7 +4669,7 @@
       <c r="O2" s="25"/>
       <c r="P2" s="25"/>
     </row>
-    <row r="3" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="26"/>
       <c r="B3" s="26"/>
       <c r="C3" s="1"/>
@@ -4605,7 +4680,7 @@
       <c r="M3" s="1"/>
       <c r="O3" s="1"/>
     </row>
-    <row r="5" spans="1:16" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
@@ -4646,7 +4721,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
@@ -4669,11 +4744,11 @@
       </c>
       <c r="G6" s="4">
         <f>COUNTIFS('V1 - Encoding and Sanitization'!$F$2:$F$36,"Compliant",'V1 - Encoding and Sanitization'!$E$2:$E$36,2)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H6" s="5">
         <f t="shared" ref="H6:H22" si="1">IF(F6=0,"",G6/F6)</f>
-        <v>0</v>
+        <v>0.15789473684210525</v>
       </c>
       <c r="I6" s="4">
         <v>3</v>
@@ -4688,14 +4763,14 @@
       </c>
       <c r="L6" s="4">
         <f>COUNTIF('V1 - Encoding and Sanitization'!$F$2:$F$36,"Compliant")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M6" s="5">
         <f t="shared" ref="M6:M22" si="3">IF(B6=0,"",L6/B6)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
         <v>15</v>
       </c>
@@ -4744,7 +4819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>16</v>
       </c>
@@ -4793,7 +4868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
         <v>17</v>
       </c>
@@ -4842,7 +4917,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>18</v>
       </c>
@@ -4891,7 +4966,7 @@
         <v>0.23076923076923078</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
         <v>19</v>
       </c>
@@ -4940,7 +5015,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
@@ -4989,7 +5064,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
         <v>21</v>
       </c>
@@ -5038,7 +5113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>22</v>
       </c>
@@ -5085,7 +5160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
         <v>24</v>
       </c>
@@ -5134,7 +5209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>25</v>
       </c>
@@ -5183,7 +5258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="6" t="s">
         <v>26</v>
       </c>
@@ -5232,7 +5307,7 @@
         <v>8.3333333333333329E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>27</v>
       </c>
@@ -5281,7 +5356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="6" t="s">
         <v>28</v>
       </c>
@@ -5330,7 +5405,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
         <v>29</v>
       </c>
@@ -5379,7 +5454,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="6" t="s">
         <v>30</v>
       </c>
@@ -5426,7 +5501,7 @@
         <v>0.11764705882352941</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>31</v>
       </c>
@@ -5473,7 +5548,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="9" t="s">
         <v>32</v>
       </c>
@@ -5499,11 +5574,11 @@
       </c>
       <c r="G23" s="10">
         <f>SUM(G6:G22)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H23" s="11">
         <f>IFERROR(AVERAGE(H6:H22),"")</f>
-        <v>1.9117647058823531E-2</v>
+        <v>2.8405572755417958E-2</v>
       </c>
       <c r="I23" s="10">
         <f>SUM(I6:I22)</f>
@@ -5519,11 +5594,11 @@
       </c>
       <c r="L23" s="10">
         <f>SUM(L6:L22)</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="M23" s="11">
         <f>IFERROR(AVERAGE(M6:M22),"")</f>
-        <v>2.5397036642711385E-2</v>
+        <v>3.1279389583887852E-2</v>
       </c>
     </row>
   </sheetData>
@@ -5589,7 +5664,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:H10"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -5601,7 +5676,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -5627,7 +5702,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>490</v>
       </c>
@@ -5641,7 +5716,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>490</v>
       </c>
@@ -5663,7 +5738,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>490</v>
       </c>
@@ -5685,7 +5760,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>490</v>
       </c>
@@ -5707,7 +5782,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="13" t="s">
         <v>498</v>
       </c>
@@ -5721,7 +5796,7 @@
       <c r="G6" s="13"/>
       <c r="H6" s="13"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
         <v>498</v>
       </c>
@@ -5743,7 +5818,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="19" t="s">
         <v>498</v>
       </c>
@@ -5765,7 +5840,7 @@
       <c r="G8" s="21"/>
       <c r="H8" s="21"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
         <v>498</v>
       </c>
@@ -5787,7 +5862,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="19" t="s">
         <v>498</v>
       </c>
@@ -5835,7 +5910,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:H44"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -5847,7 +5922,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -5873,7 +5948,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>508</v>
       </c>
@@ -5887,7 +5962,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>508</v>
       </c>
@@ -5909,7 +5984,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>508</v>
       </c>
@@ -5931,7 +6006,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="13" t="s">
         <v>514</v>
       </c>
@@ -5945,7 +6020,7 @@
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="14" t="s">
         <v>514</v>
       </c>
@@ -5967,7 +6042,7 @@
       <c r="G6" s="16"/>
       <c r="H6" s="16"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="19" t="s">
         <v>514</v>
       </c>
@@ -5989,7 +6064,7 @@
       <c r="G7" s="21"/>
       <c r="H7" s="21"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="14" t="s">
         <v>514</v>
       </c>
@@ -6011,7 +6086,7 @@
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
     </row>
-    <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="13" t="s">
         <v>522</v>
       </c>
@@ -6025,7 +6100,7 @@
       <c r="G9" s="13"/>
       <c r="H9" s="13"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="14" t="s">
         <v>522</v>
       </c>
@@ -6047,7 +6122,7 @@
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="19" t="s">
         <v>522</v>
       </c>
@@ -6069,7 +6144,7 @@
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>522</v>
       </c>
@@ -6091,7 +6166,7 @@
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="19" t="s">
         <v>522</v>
       </c>
@@ -6113,7 +6188,7 @@
       <c r="G13" s="21"/>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="14" t="s">
         <v>522</v>
       </c>
@@ -6135,7 +6210,7 @@
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
     </row>
-    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="13" t="s">
         <v>534</v>
       </c>
@@ -6149,7 +6224,7 @@
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="14" t="s">
         <v>534</v>
       </c>
@@ -6171,7 +6246,7 @@
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="19" t="s">
         <v>534</v>
       </c>
@@ -6193,7 +6268,7 @@
       <c r="G17" s="21"/>
       <c r="H17" s="21"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="14" t="s">
         <v>534</v>
       </c>
@@ -6215,7 +6290,7 @@
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="19" t="s">
         <v>534</v>
       </c>
@@ -6237,7 +6312,7 @@
       <c r="G19" s="21"/>
       <c r="H19" s="21"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="14" t="s">
         <v>534</v>
       </c>
@@ -6259,7 +6334,7 @@
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="19" t="s">
         <v>534</v>
       </c>
@@ -6281,7 +6356,7 @@
       <c r="G21" s="21"/>
       <c r="H21" s="21"/>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="14" t="s">
         <v>534</v>
       </c>
@@ -6303,7 +6378,7 @@
       <c r="G22" s="16"/>
       <c r="H22" s="16"/>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="19" t="s">
         <v>534</v>
       </c>
@@ -6325,7 +6400,7 @@
       <c r="G23" s="21"/>
       <c r="H23" s="21"/>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="14" t="s">
         <v>534</v>
       </c>
@@ -6347,7 +6422,7 @@
       <c r="G24" s="16"/>
       <c r="H24" s="16"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="19" t="s">
         <v>534</v>
       </c>
@@ -6369,7 +6444,7 @@
       <c r="G25" s="21"/>
       <c r="H25" s="21"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="14" t="s">
         <v>534</v>
       </c>
@@ -6391,7 +6466,7 @@
       <c r="G26" s="16"/>
       <c r="H26" s="16"/>
     </row>
-    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="19" t="s">
         <v>534</v>
       </c>
@@ -6413,7 +6488,7 @@
       <c r="G27" s="21"/>
       <c r="H27" s="21"/>
     </row>
-    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="14" t="s">
         <v>534</v>
       </c>
@@ -6435,7 +6510,7 @@
       <c r="G28" s="16"/>
       <c r="H28" s="16"/>
     </row>
-    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="19" t="s">
         <v>534</v>
       </c>
@@ -6457,7 +6532,7 @@
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
     </row>
-    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="14" t="s">
         <v>534</v>
       </c>
@@ -6479,7 +6554,7 @@
       <c r="G30" s="16"/>
       <c r="H30" s="16"/>
     </row>
-    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="19" t="s">
         <v>534</v>
       </c>
@@ -6501,7 +6576,7 @@
       <c r="G31" s="21"/>
       <c r="H31" s="21"/>
     </row>
-    <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="13" t="s">
         <v>568</v>
       </c>
@@ -6515,7 +6590,7 @@
       <c r="G32" s="13"/>
       <c r="H32" s="13"/>
     </row>
-    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="14" t="s">
         <v>568</v>
       </c>
@@ -6537,7 +6612,7 @@
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
     </row>
-    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="19" t="s">
         <v>568</v>
       </c>
@@ -6559,7 +6634,7 @@
       <c r="G34" s="21"/>
       <c r="H34" s="21"/>
     </row>
-    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="14" t="s">
         <v>568</v>
       </c>
@@ -6581,7 +6656,7 @@
       <c r="G35" s="16"/>
       <c r="H35" s="16"/>
     </row>
-    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="19" t="s">
         <v>568</v>
       </c>
@@ -6603,7 +6678,7 @@
       <c r="G36" s="21"/>
       <c r="H36" s="21"/>
     </row>
-    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="14" t="s">
         <v>568</v>
       </c>
@@ -6625,7 +6700,7 @@
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
     </row>
-    <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="13" t="s">
         <v>580</v>
       </c>
@@ -6639,7 +6714,7 @@
       <c r="G38" s="13"/>
       <c r="H38" s="13"/>
     </row>
-    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="14" t="s">
         <v>580</v>
       </c>
@@ -6661,7 +6736,7 @@
       <c r="G39" s="16"/>
       <c r="H39" s="16"/>
     </row>
-    <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="19" t="s">
         <v>580</v>
       </c>
@@ -6683,7 +6758,7 @@
       <c r="G40" s="21"/>
       <c r="H40" s="21"/>
     </row>
-    <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="13" t="s">
         <v>586</v>
       </c>
@@ -6697,7 +6772,7 @@
       <c r="G41" s="13"/>
       <c r="H41" s="13"/>
     </row>
-    <row r="42" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="14" t="s">
         <v>586</v>
       </c>
@@ -6719,7 +6794,7 @@
       <c r="G42" s="16"/>
       <c r="H42" s="16"/>
     </row>
-    <row r="43" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="19" t="s">
         <v>586</v>
       </c>
@@ -6741,7 +6816,7 @@
       <c r="G43" s="21"/>
       <c r="H43" s="21"/>
     </row>
-    <row r="44" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="14" t="s">
         <v>586</v>
       </c>
@@ -6789,7 +6864,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:H32"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -6801,7 +6876,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -6827,7 +6902,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>594</v>
       </c>
@@ -6841,7 +6916,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>594</v>
       </c>
@@ -6863,7 +6938,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>594</v>
       </c>
@@ -6885,7 +6960,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>594</v>
       </c>
@@ -6907,7 +6982,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>594</v>
       </c>
@@ -6929,7 +7004,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="13" t="s">
         <v>604</v>
       </c>
@@ -6943,7 +7018,7 @@
       <c r="G7" s="13"/>
       <c r="H7" s="13"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="14" t="s">
         <v>604</v>
       </c>
@@ -6965,7 +7040,7 @@
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="19" t="s">
         <v>604</v>
       </c>
@@ -6987,7 +7062,7 @@
       <c r="G9" s="21"/>
       <c r="H9" s="21"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="14" t="s">
         <v>604</v>
       </c>
@@ -7009,7 +7084,7 @@
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="19" t="s">
         <v>604</v>
       </c>
@@ -7031,7 +7106,7 @@
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>604</v>
       </c>
@@ -7053,7 +7128,7 @@
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="13" t="s">
         <v>616</v>
       </c>
@@ -7067,7 +7142,7 @@
       <c r="G13" s="13"/>
       <c r="H13" s="13"/>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="14" t="s">
         <v>616</v>
       </c>
@@ -7089,7 +7164,7 @@
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="19" t="s">
         <v>616</v>
       </c>
@@ -7111,7 +7186,7 @@
       <c r="G15" s="21"/>
       <c r="H15" s="21"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="14" t="s">
         <v>616</v>
       </c>
@@ -7133,7 +7208,7 @@
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="19" t="s">
         <v>616</v>
       </c>
@@ -7155,7 +7230,7 @@
       <c r="G17" s="21"/>
       <c r="H17" s="21"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="14" t="s">
         <v>616</v>
       </c>
@@ -7177,7 +7252,7 @@
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
     </row>
-    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="13" t="s">
         <v>628</v>
       </c>
@@ -7191,7 +7266,7 @@
       <c r="G19" s="13"/>
       <c r="H19" s="13"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="14" t="s">
         <v>628</v>
       </c>
@@ -7213,7 +7288,7 @@
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="19" t="s">
         <v>628</v>
       </c>
@@ -7235,7 +7310,7 @@
       <c r="G21" s="21"/>
       <c r="H21" s="21"/>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="14" t="s">
         <v>628</v>
       </c>
@@ -7257,7 +7332,7 @@
       <c r="G22" s="16"/>
       <c r="H22" s="16"/>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="19" t="s">
         <v>628</v>
       </c>
@@ -7279,7 +7354,7 @@
       <c r="G23" s="21"/>
       <c r="H23" s="21"/>
     </row>
-    <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="13" t="s">
         <v>638</v>
       </c>
@@ -7293,7 +7368,7 @@
       <c r="G24" s="13"/>
       <c r="H24" s="13"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="14" t="s">
         <v>638</v>
       </c>
@@ -7315,7 +7390,7 @@
       <c r="G25" s="16"/>
       <c r="H25" s="16"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="19" t="s">
         <v>638</v>
       </c>
@@ -7337,7 +7412,7 @@
       <c r="G26" s="21"/>
       <c r="H26" s="21"/>
     </row>
-    <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="13" t="s">
         <v>644</v>
       </c>
@@ -7351,7 +7426,7 @@
       <c r="G27" s="13"/>
       <c r="H27" s="13"/>
     </row>
-    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="14" t="s">
         <v>644</v>
       </c>
@@ -7373,7 +7448,7 @@
       <c r="G28" s="16"/>
       <c r="H28" s="16"/>
     </row>
-    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="19" t="s">
         <v>644</v>
       </c>
@@ -7395,7 +7470,7 @@
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
     </row>
-    <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="13" t="s">
         <v>650</v>
       </c>
@@ -7409,7 +7484,7 @@
       <c r="G30" s="13"/>
       <c r="H30" s="13"/>
     </row>
-    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="14" t="s">
         <v>650</v>
       </c>
@@ -7431,7 +7506,7 @@
       <c r="G31" s="16"/>
       <c r="H31" s="16"/>
     </row>
-    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="19" t="s">
         <v>650</v>
       </c>
@@ -7479,7 +7554,7 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -7491,7 +7566,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -7517,7 +7592,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>656</v>
       </c>
@@ -7531,7 +7606,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>656</v>
       </c>
@@ -7557,7 +7632,7 @@
         <v>946</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>656</v>
       </c>
@@ -7579,7 +7654,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>656</v>
       </c>
@@ -7601,7 +7676,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>656</v>
       </c>
@@ -7623,7 +7698,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
         <v>656</v>
       </c>
@@ -7645,7 +7720,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="13" t="s">
         <v>668</v>
       </c>
@@ -7659,7 +7734,7 @@
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
         <v>668</v>
       </c>
@@ -7685,7 +7760,7 @@
         <v>946</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="19" t="s">
         <v>668</v>
       </c>
@@ -7711,7 +7786,7 @@
         <v>946</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
         <v>674</v>
       </c>
@@ -7725,7 +7800,7 @@
       <c r="G11" s="13"/>
       <c r="H11" s="13"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>674</v>
       </c>
@@ -7751,7 +7826,7 @@
         <v>946</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="19" t="s">
         <v>674</v>
       </c>
@@ -7773,7 +7848,7 @@
       <c r="G13" s="21"/>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="14" t="s">
         <v>674</v>
       </c>
@@ -7799,7 +7874,7 @@
         <v>946</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="19" t="s">
         <v>674</v>
       </c>
@@ -7821,7 +7896,7 @@
       <c r="G15" s="21"/>
       <c r="H15" s="21"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="14" t="s">
         <v>674</v>
       </c>
@@ -7869,7 +7944,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:H26"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -7881,7 +7956,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -7907,7 +7982,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>686</v>
       </c>
@@ -7921,7 +7996,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>686</v>
       </c>
@@ -7943,7 +8018,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>686</v>
       </c>
@@ -7965,7 +8040,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>686</v>
       </c>
@@ -7987,7 +8062,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>686</v>
       </c>
@@ -8009,7 +8084,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="13" t="s">
         <v>696</v>
       </c>
@@ -8023,7 +8098,7 @@
       <c r="G7" s="13"/>
       <c r="H7" s="13"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="14" t="s">
         <v>696</v>
       </c>
@@ -8045,7 +8120,7 @@
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="19" t="s">
         <v>696</v>
       </c>
@@ -8067,7 +8142,7 @@
       <c r="G9" s="21"/>
       <c r="H9" s="21"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="14" t="s">
         <v>696</v>
       </c>
@@ -8089,7 +8164,7 @@
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="19" t="s">
         <v>696</v>
       </c>
@@ -8111,7 +8186,7 @@
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>696</v>
       </c>
@@ -8133,7 +8208,7 @@
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="19" t="s">
         <v>696</v>
       </c>
@@ -8155,7 +8230,7 @@
       <c r="G13" s="21"/>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="13" t="s">
         <v>710</v>
       </c>
@@ -8169,7 +8244,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
         <v>710</v>
       </c>
@@ -8191,7 +8266,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>710</v>
       </c>
@@ -8213,7 +8288,7 @@
       <c r="G16" s="21"/>
       <c r="H16" s="21"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="14" t="s">
         <v>710</v>
       </c>
@@ -8235,7 +8310,7 @@
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="19" t="s">
         <v>710</v>
       </c>
@@ -8257,7 +8332,7 @@
       <c r="G18" s="21"/>
       <c r="H18" s="21"/>
     </row>
-    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="13" t="s">
         <v>720</v>
       </c>
@@ -8271,7 +8346,7 @@
       <c r="G19" s="13"/>
       <c r="H19" s="13"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="14" t="s">
         <v>720</v>
       </c>
@@ -8293,7 +8368,7 @@
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="19" t="s">
         <v>720</v>
       </c>
@@ -8315,7 +8390,7 @@
       <c r="G21" s="21"/>
       <c r="H21" s="21"/>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="14" t="s">
         <v>720</v>
       </c>
@@ -8337,7 +8412,7 @@
       <c r="G22" s="16"/>
       <c r="H22" s="16"/>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="19" t="s">
         <v>720</v>
       </c>
@@ -8359,7 +8434,7 @@
       <c r="G23" s="21"/>
       <c r="H23" s="21"/>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="14" t="s">
         <v>720</v>
       </c>
@@ -8381,7 +8456,7 @@
       <c r="G24" s="16"/>
       <c r="H24" s="16"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="19" t="s">
         <v>720</v>
       </c>
@@ -8403,7 +8478,7 @@
       <c r="G25" s="21"/>
       <c r="H25" s="21"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="14" t="s">
         <v>720</v>
       </c>
@@ -8451,7 +8526,7 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:H17"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -8463,7 +8538,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -8489,7 +8564,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>736</v>
       </c>
@@ -8503,7 +8578,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>736</v>
       </c>
@@ -8527,7 +8602,7 @@
         <v>901</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>736</v>
       </c>
@@ -8551,7 +8626,7 @@
         <v>898</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="13" t="s">
         <v>742</v>
       </c>
@@ -8565,7 +8640,7 @@
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="14" t="s">
         <v>742</v>
       </c>
@@ -8587,7 +8662,7 @@
       <c r="G6" s="16"/>
       <c r="H6" s="16"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="19" t="s">
         <v>742</v>
       </c>
@@ -8609,7 +8684,7 @@
       <c r="G7" s="21"/>
       <c r="H7" s="21"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="14" t="s">
         <v>742</v>
       </c>
@@ -8631,7 +8706,7 @@
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="19" t="s">
         <v>742</v>
       </c>
@@ -8653,7 +8728,7 @@
       <c r="G9" s="21"/>
       <c r="H9" s="21"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="14" t="s">
         <v>742</v>
       </c>
@@ -8675,7 +8750,7 @@
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="19" t="s">
         <v>742</v>
       </c>
@@ -8697,7 +8772,7 @@
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>742</v>
       </c>
@@ -8719,7 +8794,7 @@
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="19" t="s">
         <v>742</v>
       </c>
@@ -8741,7 +8816,7 @@
       <c r="G13" s="21"/>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="13" t="s">
         <v>760</v>
       </c>
@@ -8755,7 +8830,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
         <v>760</v>
       </c>
@@ -8777,7 +8852,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>760</v>
       </c>
@@ -8799,7 +8874,7 @@
       <c r="G16" s="21"/>
       <c r="H16" s="21"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="14" t="s">
         <v>760</v>
       </c>
@@ -8847,7 +8922,7 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:H26"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -8859,7 +8934,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -8885,7 +8960,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>768</v>
       </c>
@@ -8899,7 +8974,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>768</v>
       </c>
@@ -8923,7 +8998,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>768</v>
       </c>
@@ -8945,7 +9020,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>768</v>
       </c>
@@ -8967,7 +9042,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>768</v>
       </c>
@@ -8989,7 +9064,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
         <v>768</v>
       </c>
@@ -9011,7 +9086,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="13" t="s">
         <v>780</v>
       </c>
@@ -9025,7 +9100,7 @@
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
         <v>780</v>
       </c>
@@ -9047,7 +9122,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="19" t="s">
         <v>780</v>
       </c>
@@ -9069,7 +9144,7 @@
       <c r="G10" s="21"/>
       <c r="H10" s="21"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="14" t="s">
         <v>780</v>
       </c>
@@ -9091,7 +9166,7 @@
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="19" t="s">
         <v>780</v>
       </c>
@@ -9113,7 +9188,7 @@
       <c r="G12" s="21"/>
       <c r="H12" s="21"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
         <v>780</v>
       </c>
@@ -9135,7 +9210,7 @@
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="13" t="s">
         <v>792</v>
       </c>
@@ -9149,7 +9224,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
         <v>792</v>
       </c>
@@ -9171,7 +9246,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>792</v>
       </c>
@@ -9193,7 +9268,7 @@
       <c r="G16" s="21"/>
       <c r="H16" s="21"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="14" t="s">
         <v>792</v>
       </c>
@@ -9215,7 +9290,7 @@
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="19" t="s">
         <v>792</v>
       </c>
@@ -9237,7 +9312,7 @@
       <c r="G18" s="21"/>
       <c r="H18" s="21"/>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="14" t="s">
         <v>792</v>
       </c>
@@ -9259,7 +9334,7 @@
       <c r="G19" s="16"/>
       <c r="H19" s="16"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="19" t="s">
         <v>792</v>
       </c>
@@ -9281,7 +9356,7 @@
       <c r="G20" s="21"/>
       <c r="H20" s="21"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="14" t="s">
         <v>792</v>
       </c>
@@ -9303,7 +9378,7 @@
       <c r="G21" s="16"/>
       <c r="H21" s="16"/>
     </row>
-    <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="13" t="s">
         <v>808</v>
       </c>
@@ -9317,7 +9392,7 @@
       <c r="G22" s="13"/>
       <c r="H22" s="13"/>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="14" t="s">
         <v>808</v>
       </c>
@@ -9339,7 +9414,7 @@
       <c r="G23" s="16"/>
       <c r="H23" s="16"/>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="19" t="s">
         <v>808</v>
       </c>
@@ -9361,7 +9436,7 @@
       <c r="G24" s="21"/>
       <c r="H24" s="21"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="14" t="s">
         <v>808</v>
       </c>
@@ -9383,7 +9458,7 @@
       <c r="G25" s="16"/>
       <c r="H25" s="16"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="19" t="s">
         <v>808</v>
       </c>
@@ -9431,7 +9506,7 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="A1:H23"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -9443,7 +9518,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -9469,7 +9544,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>818</v>
       </c>
@@ -9483,7 +9558,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>818</v>
       </c>
@@ -9509,7 +9584,7 @@
         <v>952</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="13" t="s">
         <v>822</v>
       </c>
@@ -9523,7 +9598,7 @@
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>822</v>
       </c>
@@ -9549,7 +9624,7 @@
         <v>954</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>822</v>
       </c>
@@ -9575,7 +9650,7 @@
         <v>956</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
         <v>822</v>
       </c>
@@ -9597,7 +9672,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="19" t="s">
         <v>822</v>
       </c>
@@ -9623,7 +9698,7 @@
         <v>958</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
         <v>822</v>
       </c>
@@ -9649,7 +9724,7 @@
         <v>960</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="13" t="s">
         <v>834</v>
       </c>
@@ -9663,7 +9738,7 @@
       <c r="G10" s="13"/>
       <c r="H10" s="13"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="14" t="s">
         <v>834</v>
       </c>
@@ -9689,7 +9764,7 @@
         <v>962</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="19" t="s">
         <v>834</v>
       </c>
@@ -9715,7 +9790,7 @@
         <v>958</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
         <v>834</v>
       </c>
@@ -9741,7 +9816,7 @@
         <v>958</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="19" t="s">
         <v>834</v>
       </c>
@@ -9767,7 +9842,7 @@
         <v>966</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="13" t="s">
         <v>844</v>
       </c>
@@ -9781,7 +9856,7 @@
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="14" t="s">
         <v>844</v>
       </c>
@@ -9807,7 +9882,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="19" t="s">
         <v>844</v>
       </c>
@@ -9833,7 +9908,7 @@
         <v>958</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="14" t="s">
         <v>844</v>
       </c>
@@ -9855,7 +9930,7 @@
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
     </row>
-    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="13" t="s">
         <v>852</v>
       </c>
@@ -9869,7 +9944,7 @@
       <c r="G19" s="13"/>
       <c r="H19" s="13"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="14" t="s">
         <v>852</v>
       </c>
@@ -9895,7 +9970,7 @@
         <v>960</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="19" t="s">
         <v>852</v>
       </c>
@@ -9915,7 +9990,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="14" t="s">
         <v>852</v>
       </c>
@@ -9941,7 +10016,7 @@
         <v>971</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="19" t="s">
         <v>852</v>
       </c>
@@ -9990,7 +10065,7 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -10002,7 +10077,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -10028,7 +10103,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>862</v>
       </c>
@@ -10042,7 +10117,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>862</v>
       </c>
@@ -10064,7 +10139,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>862</v>
       </c>
@@ -10086,7 +10161,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="13" t="s">
         <v>868</v>
       </c>
@@ -10100,7 +10175,7 @@
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="14" t="s">
         <v>868</v>
       </c>
@@ -10122,7 +10197,7 @@
       <c r="G6" s="16"/>
       <c r="H6" s="16"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="19" t="s">
         <v>868</v>
       </c>
@@ -10144,7 +10219,7 @@
       <c r="G7" s="21"/>
       <c r="H7" s="21"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="14" t="s">
         <v>868</v>
       </c>
@@ -10166,7 +10241,7 @@
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="19" t="s">
         <v>868</v>
       </c>
@@ -10188,7 +10263,7 @@
       <c r="G9" s="21"/>
       <c r="H9" s="21"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="14" t="s">
         <v>868</v>
       </c>
@@ -10210,7 +10285,7 @@
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="19" t="s">
         <v>868</v>
       </c>
@@ -10232,7 +10307,7 @@
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>868</v>
       </c>
@@ -10254,7 +10329,7 @@
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="19" t="s">
         <v>868</v>
       </c>
@@ -10276,7 +10351,7 @@
       <c r="G13" s="21"/>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="13" t="s">
         <v>886</v>
       </c>
@@ -10290,7 +10365,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
         <v>886</v>
       </c>
@@ -10312,7 +10387,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>886</v>
       </c>
@@ -10360,7 +10435,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H36"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -10372,7 +10447,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -10398,7 +10473,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>41</v>
       </c>
@@ -10412,7 +10487,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>41</v>
       </c>
@@ -10434,7 +10509,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>41</v>
       </c>
@@ -10460,7 +10535,7 @@
         <v>937</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="13" t="s">
         <v>48</v>
       </c>
@@ -10474,7 +10549,7 @@
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="14" t="s">
         <v>48</v>
       </c>
@@ -10500,7 +10575,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="19" t="s">
         <v>48</v>
       </c>
@@ -10517,12 +10592,16 @@
         <v>1</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G7" s="21"/>
-      <c r="H7" s="21"/>
-    </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G7" s="21" t="s">
+        <v>972</v>
+      </c>
+      <c r="H7" s="21" t="s">
+        <v>918</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="14" t="s">
         <v>48</v>
       </c>
@@ -10539,12 +10618,16 @@
         <v>1</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
-    </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G8" s="16" t="s">
+        <v>973</v>
+      </c>
+      <c r="H8" s="16" t="s">
+        <v>918</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="19" t="s">
         <v>48</v>
       </c>
@@ -10570,7 +10653,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="14" t="s">
         <v>48</v>
       </c>
@@ -10596,7 +10679,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="19" t="s">
         <v>48</v>
       </c>
@@ -10613,12 +10696,12 @@
         <v>2</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>45</v>
+        <v>894</v>
       </c>
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>48</v>
       </c>
@@ -10635,12 +10718,12 @@
         <v>2</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>45</v>
+        <v>894</v>
       </c>
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="19" t="s">
         <v>48</v>
       </c>
@@ -10657,12 +10740,12 @@
         <v>2</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>45</v>
+        <v>894</v>
       </c>
       <c r="G13" s="21"/>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="14" t="s">
         <v>48</v>
       </c>
@@ -10688,7 +10771,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="19" t="s">
         <v>48</v>
       </c>
@@ -10710,7 +10793,7 @@
       <c r="G15" s="21"/>
       <c r="H15" s="21"/>
     </row>
-    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="13" t="s">
         <v>70</v>
       </c>
@@ -10724,7 +10807,7 @@
       <c r="G16" s="13"/>
       <c r="H16" s="13"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="14" t="s">
         <v>70</v>
       </c>
@@ -10750,7 +10833,7 @@
         <v>937</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="19" t="s">
         <v>70</v>
       </c>
@@ -10767,12 +10850,16 @@
         <v>1</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G18" s="21"/>
-      <c r="H18" s="21"/>
-    </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G18" s="21" t="s">
+        <v>974</v>
+      </c>
+      <c r="H18" s="21" t="s">
+        <v>918</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="14" t="s">
         <v>70</v>
       </c>
@@ -10798,7 +10885,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="19" t="s">
         <v>70</v>
       </c>
@@ -10820,7 +10907,7 @@
       <c r="G20" s="21"/>
       <c r="H20" s="21"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="14" t="s">
         <v>70</v>
       </c>
@@ -10837,12 +10924,16 @@
         <v>2</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G21" s="16"/>
-      <c r="H21" s="16"/>
-    </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G21" s="16" t="s">
+        <v>975</v>
+      </c>
+      <c r="H21" s="16" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="19" t="s">
         <v>70</v>
       </c>
@@ -10864,7 +10955,7 @@
       <c r="G22" s="21"/>
       <c r="H22" s="21"/>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="14" t="s">
         <v>70</v>
       </c>
@@ -10886,7 +10977,7 @@
       <c r="G23" s="16"/>
       <c r="H23" s="16"/>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="19" t="s">
         <v>70</v>
       </c>
@@ -10908,7 +10999,7 @@
       <c r="G24" s="21"/>
       <c r="H24" s="21"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="14" t="s">
         <v>70</v>
       </c>
@@ -10934,7 +11025,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="19" t="s">
         <v>70</v>
       </c>
@@ -10956,7 +11047,7 @@
       <c r="G26" s="21"/>
       <c r="H26" s="21"/>
     </row>
-    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="14" t="s">
         <v>70</v>
       </c>
@@ -10978,7 +11069,7 @@
       <c r="G27" s="16"/>
       <c r="H27" s="16"/>
     </row>
-    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="19" t="s">
         <v>70</v>
       </c>
@@ -11000,7 +11091,7 @@
       <c r="G28" s="21"/>
       <c r="H28" s="21"/>
     </row>
-    <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="13" t="s">
         <v>96</v>
       </c>
@@ -11014,7 +11105,7 @@
       <c r="G29" s="13"/>
       <c r="H29" s="13"/>
     </row>
-    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="14" t="s">
         <v>96</v>
       </c>
@@ -11031,12 +11122,16 @@
         <v>2</v>
       </c>
       <c r="F30" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G30" s="16"/>
-      <c r="H30" s="16"/>
-    </row>
-    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>916</v>
+      </c>
+      <c r="G30" s="16" t="s">
+        <v>977</v>
+      </c>
+      <c r="H30" s="16" t="s">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="19" t="s">
         <v>96</v>
       </c>
@@ -11053,12 +11148,16 @@
         <v>2</v>
       </c>
       <c r="F31" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G31" s="21"/>
-      <c r="H31" s="21"/>
-    </row>
-    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>916</v>
+      </c>
+      <c r="G31" s="21" t="s">
+        <v>979</v>
+      </c>
+      <c r="H31" s="21" t="s">
+        <v>918</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="14" t="s">
         <v>96</v>
       </c>
@@ -11075,12 +11174,16 @@
         <v>2</v>
       </c>
       <c r="F32" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G32" s="16"/>
-      <c r="H32" s="16"/>
-    </row>
-    <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+        <v>916</v>
+      </c>
+      <c r="G32" s="16" t="s">
+        <v>980</v>
+      </c>
+      <c r="H32" s="16" t="s">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="13" t="s">
         <v>104</v>
       </c>
@@ -11094,7 +11197,7 @@
       <c r="G33" s="13"/>
       <c r="H33" s="13"/>
     </row>
-    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="14" t="s">
         <v>104</v>
       </c>
@@ -11116,7 +11219,7 @@
       <c r="G34" s="16"/>
       <c r="H34" s="16"/>
     </row>
-    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="19" t="s">
         <v>104</v>
       </c>
@@ -11133,12 +11236,16 @@
         <v>2</v>
       </c>
       <c r="F35" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G35" s="21"/>
-      <c r="H35" s="21"/>
-    </row>
-    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G35" s="21" t="s">
+        <v>976</v>
+      </c>
+      <c r="H35" s="21" t="s">
+        <v>918</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="14" t="s">
         <v>104</v>
       </c>
@@ -11186,7 +11293,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -11198,7 +11305,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -11224,7 +11331,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>112</v>
       </c>
@@ -11238,7 +11345,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>112</v>
       </c>
@@ -11262,7 +11369,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>112</v>
       </c>
@@ -11279,12 +11386,16 @@
         <v>2</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
-    </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G4" s="21" t="s">
+        <v>981</v>
+      </c>
+      <c r="H4" s="21" t="s">
+        <v>982</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>112</v>
       </c>
@@ -11301,12 +11412,16 @@
         <v>2</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
-    </row>
-    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>983</v>
+      </c>
+      <c r="H5" s="16" t="s">
+        <v>984</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="13" t="s">
         <v>120</v>
       </c>
@@ -11320,7 +11435,7 @@
       <c r="G6" s="13"/>
       <c r="H6" s="13"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
         <v>120</v>
       </c>
@@ -11337,12 +11452,16 @@
         <v>1</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G7" s="16"/>
-      <c r="H7" s="16"/>
-    </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>985</v>
+      </c>
+      <c r="H7" s="16" t="s">
+        <v>918</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="19" t="s">
         <v>120</v>
       </c>
@@ -11359,12 +11478,16 @@
         <v>1</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G8" s="21"/>
-      <c r="H8" s="21"/>
-    </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G8" s="21" t="s">
+        <v>986</v>
+      </c>
+      <c r="H8" s="21" t="s">
+        <v>987</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
         <v>120</v>
       </c>
@@ -11381,12 +11504,16 @@
         <v>2</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G9" s="16"/>
-      <c r="H9" s="16"/>
-    </row>
-    <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G9" s="16" t="s">
+        <v>988</v>
+      </c>
+      <c r="H9" s="16" t="s">
+        <v>930</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="13" t="s">
         <v>128</v>
       </c>
@@ -11400,7 +11527,7 @@
       <c r="G10" s="13"/>
       <c r="H10" s="13"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="14" t="s">
         <v>128</v>
       </c>
@@ -11419,10 +11546,14 @@
       <c r="F11" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="G11" s="16"/>
-      <c r="H11" s="16"/>
-    </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G11" s="16" t="s">
+        <v>989</v>
+      </c>
+      <c r="H11" s="16" t="s">
+        <v>932</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="19" t="s">
         <v>128</v>
       </c>
@@ -11441,10 +11572,14 @@
       <c r="F12" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="G12" s="21"/>
-      <c r="H12" s="21"/>
-    </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G12" s="21" t="s">
+        <v>990</v>
+      </c>
+      <c r="H12" s="21" t="s">
+        <v>991</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
         <v>128</v>
       </c>
@@ -11463,10 +11598,14 @@
       <c r="F13" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="G13" s="16"/>
-      <c r="H13" s="16"/>
-    </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G13" s="16" t="s">
+        <v>992</v>
+      </c>
+      <c r="H13" s="16" t="s">
+        <v>993</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="19" t="s">
         <v>128</v>
       </c>
@@ -11488,7 +11627,7 @@
       <c r="G14" s="21"/>
       <c r="H14" s="21"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
         <v>128</v>
       </c>
@@ -11505,12 +11644,16 @@
         <v>3</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G15" s="16"/>
-      <c r="H15" s="16"/>
-    </row>
-    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G15" s="16" t="s">
+        <v>996</v>
+      </c>
+      <c r="H15" s="16" t="s">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="13" t="s">
         <v>140</v>
       </c>
@@ -11524,7 +11667,7 @@
       <c r="G16" s="13"/>
       <c r="H16" s="13"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="14" t="s">
         <v>140</v>
       </c>
@@ -11541,12 +11684,16 @@
         <v>2</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G17" s="16"/>
-      <c r="H17" s="16"/>
-    </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G17" s="16" t="s">
+        <v>994</v>
+      </c>
+      <c r="H17" s="16" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="19" t="s">
         <v>140</v>
       </c>
@@ -11594,7 +11741,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H39"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -11606,7 +11753,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -11632,7 +11779,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>146</v>
       </c>
@@ -11646,7 +11793,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>146</v>
       </c>
@@ -11670,7 +11817,7 @@
       </c>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="13" t="s">
         <v>150</v>
       </c>
@@ -11684,7 +11831,7 @@
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>150</v>
       </c>
@@ -11706,7 +11853,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>150</v>
       </c>
@@ -11728,7 +11875,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
         <v>150</v>
       </c>
@@ -11750,7 +11897,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="13" t="s">
         <v>158</v>
       </c>
@@ -11764,7 +11911,7 @@
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
         <v>158</v>
       </c>
@@ -11786,7 +11933,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="19" t="s">
         <v>158</v>
       </c>
@@ -11808,7 +11955,7 @@
       <c r="G10" s="21"/>
       <c r="H10" s="21"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="14" t="s">
         <v>158</v>
       </c>
@@ -11830,7 +11977,7 @@
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="19" t="s">
         <v>158</v>
       </c>
@@ -11852,7 +11999,7 @@
       <c r="G12" s="21"/>
       <c r="H12" s="21"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
         <v>158</v>
       </c>
@@ -11874,7 +12021,7 @@
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="13" t="s">
         <v>170</v>
       </c>
@@ -11888,7 +12035,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
         <v>170</v>
       </c>
@@ -11910,7 +12057,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>170</v>
       </c>
@@ -11932,7 +12079,7 @@
       <c r="G16" s="21"/>
       <c r="H16" s="21"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="14" t="s">
         <v>170</v>
       </c>
@@ -11954,7 +12101,7 @@
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="19" t="s">
         <v>170</v>
       </c>
@@ -11976,7 +12123,7 @@
       <c r="G18" s="21"/>
       <c r="H18" s="21"/>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="14" t="s">
         <v>170</v>
       </c>
@@ -11998,7 +12145,7 @@
       <c r="G19" s="16"/>
       <c r="H19" s="16"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="19" t="s">
         <v>170</v>
       </c>
@@ -12020,7 +12167,7 @@
       <c r="G20" s="21"/>
       <c r="H20" s="21"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="14" t="s">
         <v>170</v>
       </c>
@@ -12042,7 +12189,7 @@
       <c r="G21" s="16"/>
       <c r="H21" s="16"/>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="19" t="s">
         <v>170</v>
       </c>
@@ -12064,7 +12211,7 @@
       <c r="G22" s="21"/>
       <c r="H22" s="21"/>
     </row>
-    <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="13" t="s">
         <v>188</v>
       </c>
@@ -12078,7 +12225,7 @@
       <c r="G23" s="13"/>
       <c r="H23" s="13"/>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="14" t="s">
         <v>188</v>
       </c>
@@ -12100,7 +12247,7 @@
       <c r="G24" s="16"/>
       <c r="H24" s="16"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="19" t="s">
         <v>188</v>
       </c>
@@ -12122,7 +12269,7 @@
       <c r="G25" s="21"/>
       <c r="H25" s="21"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="14" t="s">
         <v>188</v>
       </c>
@@ -12144,7 +12291,7 @@
       <c r="G26" s="16"/>
       <c r="H26" s="16"/>
     </row>
-    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="19" t="s">
         <v>188</v>
       </c>
@@ -12166,7 +12313,7 @@
       <c r="G27" s="21"/>
       <c r="H27" s="21"/>
     </row>
-    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="14" t="s">
         <v>188</v>
       </c>
@@ -12188,7 +12335,7 @@
       <c r="G28" s="16"/>
       <c r="H28" s="16"/>
     </row>
-    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="19" t="s">
         <v>188</v>
       </c>
@@ -12210,7 +12357,7 @@
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
     </row>
-    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="14" t="s">
         <v>188</v>
       </c>
@@ -12232,7 +12379,7 @@
       <c r="G30" s="16"/>
       <c r="H30" s="16"/>
     </row>
-    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="19" t="s">
         <v>188</v>
       </c>
@@ -12254,7 +12401,7 @@
       <c r="G31" s="21"/>
       <c r="H31" s="21"/>
     </row>
-    <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="13" t="s">
         <v>206</v>
       </c>
@@ -12268,7 +12415,7 @@
       <c r="G32" s="13"/>
       <c r="H32" s="13"/>
     </row>
-    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="14" t="s">
         <v>206</v>
       </c>
@@ -12290,7 +12437,7 @@
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
     </row>
-    <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="13" t="s">
         <v>210</v>
       </c>
@@ -12304,7 +12451,7 @@
       <c r="G34" s="13"/>
       <c r="H34" s="13"/>
     </row>
-    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="14" t="s">
         <v>210</v>
       </c>
@@ -12326,7 +12473,7 @@
       <c r="G35" s="16"/>
       <c r="H35" s="16"/>
     </row>
-    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="19" t="s">
         <v>210</v>
       </c>
@@ -12348,7 +12495,7 @@
       <c r="G36" s="21"/>
       <c r="H36" s="21"/>
     </row>
-    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="14" t="s">
         <v>210</v>
       </c>
@@ -12370,7 +12517,7 @@
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
     </row>
-    <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="19" t="s">
         <v>210</v>
       </c>
@@ -12392,7 +12539,7 @@
       <c r="G38" s="21"/>
       <c r="H38" s="21"/>
     </row>
-    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="14" t="s">
         <v>210</v>
       </c>
@@ -12440,7 +12587,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -12452,7 +12599,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -12478,7 +12625,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>222</v>
       </c>
@@ -12492,7 +12639,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>222</v>
       </c>
@@ -12514,7 +12661,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>222</v>
       </c>
@@ -12536,7 +12683,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>222</v>
       </c>
@@ -12558,7 +12705,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>222</v>
       </c>
@@ -12580,7 +12727,7 @@
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
         <v>222</v>
       </c>
@@ -12602,7 +12749,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="13" t="s">
         <v>234</v>
       </c>
@@ -12616,7 +12763,7 @@
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
         <v>234</v>
       </c>
@@ -12638,7 +12785,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="19" t="s">
         <v>234</v>
       </c>
@@ -12660,7 +12807,7 @@
       <c r="G10" s="21"/>
       <c r="H10" s="21"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="14" t="s">
         <v>234</v>
       </c>
@@ -12682,7 +12829,7 @@
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="19" t="s">
         <v>234</v>
       </c>
@@ -12704,7 +12851,7 @@
       <c r="G12" s="21"/>
       <c r="H12" s="21"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
         <v>234</v>
       </c>
@@ -12726,7 +12873,7 @@
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="13" t="s">
         <v>246</v>
       </c>
@@ -12740,7 +12887,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
         <v>246</v>
       </c>
@@ -12762,7 +12909,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>246</v>
       </c>
@@ -12784,7 +12931,7 @@
       <c r="G16" s="21"/>
       <c r="H16" s="21"/>
     </row>
-    <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="13" t="s">
         <v>252</v>
       </c>
@@ -12798,7 +12945,7 @@
       <c r="G17" s="13"/>
       <c r="H17" s="13"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="14" t="s">
         <v>252</v>
       </c>
@@ -12820,7 +12967,7 @@
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="19" t="s">
         <v>252</v>
       </c>
@@ -12842,7 +12989,7 @@
       <c r="G19" s="21"/>
       <c r="H19" s="21"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="14" t="s">
         <v>252</v>
       </c>
@@ -12864,7 +13011,7 @@
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="19" t="s">
         <v>252</v>
       </c>
@@ -12912,7 +13059,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -12924,7 +13071,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -12950,7 +13097,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>262</v>
       </c>
@@ -12964,7 +13111,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>262</v>
       </c>
@@ -12990,7 +13137,7 @@
         <v>896</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="13" t="s">
         <v>266</v>
       </c>
@@ -13004,7 +13151,7 @@
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>266</v>
       </c>
@@ -13028,7 +13175,7 @@
       </c>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>266</v>
       </c>
@@ -13054,7 +13201,7 @@
         <v>917</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
         <v>266</v>
       </c>
@@ -13080,7 +13227,7 @@
         <v>917</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="19" t="s">
         <v>266</v>
       </c>
@@ -13104,7 +13251,7 @@
       </c>
       <c r="H8" s="21"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
         <v>266</v>
       </c>
@@ -13130,7 +13277,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="19" t="s">
         <v>266</v>
       </c>
@@ -13156,7 +13303,7 @@
         <v>921</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
         <v>280</v>
       </c>
@@ -13170,7 +13317,7 @@
       <c r="G11" s="13"/>
       <c r="H11" s="13"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>280</v>
       </c>
@@ -13194,7 +13341,7 @@
       </c>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="19" t="s">
         <v>280</v>
       </c>
@@ -13218,7 +13365,7 @@
       </c>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="14" t="s">
         <v>280</v>
       </c>
@@ -13244,7 +13391,7 @@
         <v>920</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="13" t="s">
         <v>288</v>
       </c>
@@ -13258,7 +13405,7 @@
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="14" t="s">
         <v>288</v>
       </c>
@@ -13284,7 +13431,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="19" t="s">
         <v>288</v>
       </c>
@@ -13310,7 +13457,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="14" t="s">
         <v>288</v>
       </c>
@@ -13362,7 +13509,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:H56"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -13374,7 +13521,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -13400,7 +13547,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>296</v>
       </c>
@@ -13414,7 +13561,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>296</v>
       </c>
@@ -13436,7 +13583,7 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>296</v>
       </c>
@@ -13458,7 +13605,7 @@
       <c r="G4" s="21"/>
       <c r="H4" s="21"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>296</v>
       </c>
@@ -13480,7 +13627,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="13" t="s">
         <v>304</v>
       </c>
@@ -13494,7 +13641,7 @@
       <c r="G6" s="13"/>
       <c r="H6" s="13"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
         <v>304</v>
       </c>
@@ -13516,7 +13663,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="19" t="s">
         <v>304</v>
       </c>
@@ -13538,7 +13685,7 @@
       <c r="G8" s="21"/>
       <c r="H8" s="21"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
         <v>304</v>
       </c>
@@ -13560,7 +13707,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="19" t="s">
         <v>304</v>
       </c>
@@ -13582,7 +13729,7 @@
       <c r="G10" s="21"/>
       <c r="H10" s="21"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="14" t="s">
         <v>304</v>
       </c>
@@ -13604,7 +13751,7 @@
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="19" t="s">
         <v>304</v>
       </c>
@@ -13626,7 +13773,7 @@
       <c r="G12" s="21"/>
       <c r="H12" s="21"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
         <v>304</v>
       </c>
@@ -13648,7 +13795,7 @@
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="19" t="s">
         <v>304</v>
       </c>
@@ -13670,7 +13817,7 @@
       <c r="G14" s="21"/>
       <c r="H14" s="21"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
         <v>304</v>
       </c>
@@ -13692,7 +13839,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>304</v>
       </c>
@@ -13714,7 +13861,7 @@
       <c r="G16" s="21"/>
       <c r="H16" s="21"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="14" t="s">
         <v>304</v>
       </c>
@@ -13736,7 +13883,7 @@
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="19" t="s">
         <v>304</v>
       </c>
@@ -13758,7 +13905,7 @@
       <c r="G18" s="21"/>
       <c r="H18" s="21"/>
     </row>
-    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="13" t="s">
         <v>330</v>
       </c>
@@ -13772,7 +13919,7 @@
       <c r="G19" s="13"/>
       <c r="H19" s="13"/>
     </row>
-    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="14" t="s">
         <v>330</v>
       </c>
@@ -13794,7 +13941,7 @@
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="19" t="s">
         <v>330</v>
       </c>
@@ -13816,7 +13963,7 @@
       <c r="G21" s="21"/>
       <c r="H21" s="21"/>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="14" t="s">
         <v>330</v>
       </c>
@@ -13838,7 +13985,7 @@
       <c r="G22" s="16"/>
       <c r="H22" s="16"/>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="19" t="s">
         <v>330</v>
       </c>
@@ -13860,7 +14007,7 @@
       <c r="G23" s="21"/>
       <c r="H23" s="21"/>
     </row>
-    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="14" t="s">
         <v>330</v>
       </c>
@@ -13882,7 +14029,7 @@
       <c r="G24" s="16"/>
       <c r="H24" s="16"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="19" t="s">
         <v>330</v>
       </c>
@@ -13904,7 +14051,7 @@
       <c r="G25" s="21"/>
       <c r="H25" s="21"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="14" t="s">
         <v>330</v>
       </c>
@@ -13926,7 +14073,7 @@
       <c r="G26" s="16"/>
       <c r="H26" s="16"/>
     </row>
-    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="19" t="s">
         <v>330</v>
       </c>
@@ -13948,7 +14095,7 @@
       <c r="G27" s="21"/>
       <c r="H27" s="21"/>
     </row>
-    <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="13" t="s">
         <v>348</v>
       </c>
@@ -13962,7 +14109,7 @@
       <c r="G28" s="13"/>
       <c r="H28" s="13"/>
     </row>
-    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="14" t="s">
         <v>348</v>
       </c>
@@ -13984,7 +14131,7 @@
       <c r="G29" s="16"/>
       <c r="H29" s="16"/>
     </row>
-    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="19" t="s">
         <v>348</v>
       </c>
@@ -14006,7 +14153,7 @@
       <c r="G30" s="21"/>
       <c r="H30" s="21"/>
     </row>
-    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="14" t="s">
         <v>348</v>
       </c>
@@ -14028,7 +14175,7 @@
       <c r="G31" s="16"/>
       <c r="H31" s="16"/>
     </row>
-    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="19" t="s">
         <v>348</v>
       </c>
@@ -14050,7 +14197,7 @@
       <c r="G32" s="21"/>
       <c r="H32" s="21"/>
     </row>
-    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="14" t="s">
         <v>348</v>
       </c>
@@ -14072,7 +14219,7 @@
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
     </row>
-    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="19" t="s">
         <v>348</v>
       </c>
@@ -14094,7 +14241,7 @@
       <c r="G34" s="21"/>
       <c r="H34" s="21"/>
     </row>
-    <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="13" t="s">
         <v>362</v>
       </c>
@@ -14108,7 +14255,7 @@
       <c r="G35" s="13"/>
       <c r="H35" s="13"/>
     </row>
-    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="14" t="s">
         <v>362</v>
       </c>
@@ -14130,7 +14277,7 @@
       <c r="G36" s="16"/>
       <c r="H36" s="16"/>
     </row>
-    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="19" t="s">
         <v>362</v>
       </c>
@@ -14152,7 +14299,7 @@
       <c r="G37" s="21"/>
       <c r="H37" s="21"/>
     </row>
-    <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="14" t="s">
         <v>362</v>
       </c>
@@ -14174,7 +14321,7 @@
       <c r="G38" s="16"/>
       <c r="H38" s="16"/>
     </row>
-    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="19" t="s">
         <v>362</v>
       </c>
@@ -14196,7 +14343,7 @@
       <c r="G39" s="21"/>
       <c r="H39" s="21"/>
     </row>
-    <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="14" t="s">
         <v>362</v>
       </c>
@@ -14218,7 +14365,7 @@
       <c r="G40" s="16"/>
       <c r="H40" s="16"/>
     </row>
-    <row r="41" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="19" t="s">
         <v>362</v>
       </c>
@@ -14240,7 +14387,7 @@
       <c r="G41" s="21"/>
       <c r="H41" s="21"/>
     </row>
-    <row r="42" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="14" t="s">
         <v>362</v>
       </c>
@@ -14262,7 +14409,7 @@
       <c r="G42" s="16"/>
       <c r="H42" s="16"/>
     </row>
-    <row r="43" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="19" t="s">
         <v>362</v>
       </c>
@@ -14284,7 +14431,7 @@
       <c r="G43" s="21"/>
       <c r="H43" s="21"/>
     </row>
-    <row r="44" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="13" t="s">
         <v>380</v>
       </c>
@@ -14298,7 +14445,7 @@
       <c r="G44" s="13"/>
       <c r="H44" s="13"/>
     </row>
-    <row r="45" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="14" t="s">
         <v>380</v>
       </c>
@@ -14320,7 +14467,7 @@
       <c r="G45" s="16"/>
       <c r="H45" s="16"/>
     </row>
-    <row r="46" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="19" t="s">
         <v>380</v>
       </c>
@@ -14342,7 +14489,7 @@
       <c r="G46" s="21"/>
       <c r="H46" s="21"/>
     </row>
-    <row r="47" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="14" t="s">
         <v>380</v>
       </c>
@@ -14364,7 +14511,7 @@
       <c r="G47" s="16"/>
       <c r="H47" s="16"/>
     </row>
-    <row r="48" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="19" t="s">
         <v>380</v>
       </c>
@@ -14386,7 +14533,7 @@
       <c r="G48" s="21"/>
       <c r="H48" s="21"/>
     </row>
-    <row r="49" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="13" t="s">
         <v>390</v>
       </c>
@@ -14400,7 +14547,7 @@
       <c r="G49" s="13"/>
       <c r="H49" s="13"/>
     </row>
-    <row r="50" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="14" t="s">
         <v>390</v>
       </c>
@@ -14422,7 +14569,7 @@
       <c r="G50" s="16"/>
       <c r="H50" s="16"/>
     </row>
-    <row r="51" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="19" t="s">
         <v>390</v>
       </c>
@@ -14444,7 +14591,7 @@
       <c r="G51" s="21"/>
       <c r="H51" s="21"/>
     </row>
-    <row r="52" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="13" t="s">
         <v>396</v>
       </c>
@@ -14458,7 +14605,7 @@
       <c r="G52" s="13"/>
       <c r="H52" s="13"/>
     </row>
-    <row r="53" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="14" t="s">
         <v>396</v>
       </c>
@@ -14480,7 +14627,7 @@
       <c r="G53" s="16"/>
       <c r="H53" s="16"/>
     </row>
-    <row r="54" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="19" t="s">
         <v>396</v>
       </c>
@@ -14502,7 +14649,7 @@
       <c r="G54" s="21"/>
       <c r="H54" s="21"/>
     </row>
-    <row r="55" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="14" t="s">
         <v>396</v>
       </c>
@@ -14524,7 +14671,7 @@
       <c r="G55" s="16"/>
       <c r="H55" s="16"/>
     </row>
-    <row r="56" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="19" t="s">
         <v>396</v>
       </c>
@@ -14572,7 +14719,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:H26"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -14584,7 +14731,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -14610,7 +14757,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>406</v>
       </c>
@@ -14624,7 +14771,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>406</v>
       </c>
@@ -14648,7 +14795,7 @@
         <v>899</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>406</v>
       </c>
@@ -14672,7 +14819,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>406</v>
       </c>
@@ -14694,7 +14841,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="13" t="s">
         <v>414</v>
       </c>
@@ -14708,7 +14855,7 @@
       <c r="G6" s="13"/>
       <c r="H6" s="13"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
         <v>414</v>
       </c>
@@ -14730,7 +14877,7 @@
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="19" t="s">
         <v>414</v>
       </c>
@@ -14752,7 +14899,7 @@
       <c r="G8" s="21"/>
       <c r="H8" s="21"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
         <v>414</v>
       </c>
@@ -14774,7 +14921,7 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="19" t="s">
         <v>414</v>
       </c>
@@ -14796,7 +14943,7 @@
       <c r="G10" s="21"/>
       <c r="H10" s="21"/>
     </row>
-    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
         <v>424</v>
       </c>
@@ -14810,7 +14957,7 @@
       <c r="G11" s="13"/>
       <c r="H11" s="13"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>424</v>
       </c>
@@ -14832,7 +14979,7 @@
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="19" t="s">
         <v>424</v>
       </c>
@@ -14854,7 +15001,7 @@
       <c r="G13" s="21"/>
       <c r="H13" s="21"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="13" t="s">
         <v>430</v>
       </c>
@@ -14868,7 +15015,7 @@
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
         <v>430</v>
       </c>
@@ -14890,7 +15037,7 @@
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>430</v>
       </c>
@@ -14912,7 +15059,7 @@
       <c r="G16" s="21"/>
       <c r="H16" s="21"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="14" t="s">
         <v>430</v>
       </c>
@@ -14934,7 +15081,7 @@
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="19" t="s">
         <v>430</v>
       </c>
@@ -14956,7 +15103,7 @@
       <c r="G18" s="21"/>
       <c r="H18" s="21"/>
     </row>
-    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="14" t="s">
         <v>430</v>
       </c>
@@ -14978,7 +15125,7 @@
       <c r="G19" s="16"/>
       <c r="H19" s="16"/>
     </row>
-    <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="13" t="s">
         <v>442</v>
       </c>
@@ -14992,7 +15139,7 @@
       <c r="G20" s="13"/>
       <c r="H20" s="13"/>
     </row>
-    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="14" t="s">
         <v>442</v>
       </c>
@@ -15014,7 +15161,7 @@
       <c r="G21" s="16"/>
       <c r="H21" s="16"/>
     </row>
-    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="19" t="s">
         <v>442</v>
       </c>
@@ -15036,7 +15183,7 @@
       <c r="G22" s="21"/>
       <c r="H22" s="21"/>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="14" t="s">
         <v>442</v>
       </c>
@@ -15058,7 +15205,7 @@
       <c r="G23" s="16"/>
       <c r="H23" s="16"/>
     </row>
-    <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="13" t="s">
         <v>450</v>
       </c>
@@ -15072,7 +15219,7 @@
       <c r="G24" s="13"/>
       <c r="H24" s="13"/>
     </row>
-    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="14" t="s">
         <v>450</v>
       </c>
@@ -15094,7 +15241,7 @@
       <c r="G25" s="16"/>
       <c r="H25" s="16"/>
     </row>
-    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="19" t="s">
         <v>450</v>
       </c>
@@ -15142,7 +15289,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -15154,7 +15301,7 @@
     <col min="8" max="8" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
@@ -15180,7 +15327,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>456</v>
       </c>
@@ -15194,7 +15341,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>456</v>
       </c>
@@ -15220,7 +15367,7 @@
         <v>924</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>456</v>
       </c>
@@ -15246,7 +15393,7 @@
         <v>925</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>456</v>
       </c>
@@ -15268,7 +15415,7 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>456</v>
       </c>
@@ -15292,7 +15439,7 @@
       </c>
       <c r="H6" s="21"/>
     </row>
-    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="13" t="s">
         <v>466</v>
       </c>
@@ -15306,7 +15453,7 @@
       <c r="G7" s="13"/>
       <c r="H7" s="13"/>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="14" t="s">
         <v>466</v>
       </c>
@@ -15332,7 +15479,7 @@
         <v>929</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="19" t="s">
         <v>466</v>
       </c>
@@ -15358,7 +15505,7 @@
         <v>930</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="14" t="s">
         <v>466</v>
       </c>
@@ -15380,7 +15527,7 @@
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="19" t="s">
         <v>466</v>
       </c>
@@ -15402,7 +15549,7 @@
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
     </row>
-    <row r="12" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="13" t="s">
         <v>476</v>
       </c>
@@ -15416,7 +15563,7 @@
       <c r="G12" s="13"/>
       <c r="H12" s="13"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
         <v>476</v>
       </c>
@@ -15442,7 +15589,7 @@
         <v>932</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="19" t="s">
         <v>476</v>
       </c>
@@ -15464,7 +15611,7 @@
       <c r="G14" s="21"/>
       <c r="H14" s="21"/>
     </row>
-    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
         <v>476</v>
       </c>
@@ -15490,7 +15637,7 @@
         <v>930</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="13" t="s">
         <v>484</v>
       </c>
@@ -15504,7 +15651,7 @@
       <c r="G16" s="13"/>
       <c r="H16" s="13"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="14" t="s">
         <v>484</v>
       </c>
@@ -15526,7 +15673,7 @@
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
     </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="19" t="s">
         <v>484</v>
       </c>

</xml_diff>